<commit_message>
feat: update Design sample
</commit_message>
<xml_diff>
--- a/public/design/sample/Design sample.xlsx
+++ b/public/design/sample/Design sample.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ShaoxiongEltonHu\Documents\work_update\100si_model_data\MU Box\MU Box Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ShaoxiongEltonHu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA10B1D-3A19-482F-9A93-864E4F557935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD78C615-D2ED-4078-8145-A778BA73233E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{24AD115F-7A1E-4F6E-9165-B99BF6AE44BA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>Electrolyte code</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t>Average CE (45C)</t>
-  </si>
-  <si>
-    <t>NCM811</t>
   </si>
   <si>
     <t>Solvent 4</t>
@@ -165,37 +162,10 @@
     <t>Cell performance</t>
   </si>
   <si>
-    <t>H2</t>
-  </si>
-  <si>
-    <t>12 Si-C</t>
-  </si>
-  <si>
-    <t>O=C1OCCO1</t>
-  </si>
-  <si>
-    <t>CCOC(=O)OC</t>
-  </si>
-  <si>
-    <t>CCOC(=O)OCC</t>
-  </si>
-  <si>
-    <t>F[P-](F)(F)(F)(F)F.[Li+]</t>
-  </si>
-  <si>
-    <t>O=S(=O)(F)[N-]S(=O)(=O)F.[Li+]</t>
-  </si>
-  <si>
-    <t>O=c1occo1</t>
-  </si>
-  <si>
-    <t>O=P([O-])(F)F.[Li+]</t>
-  </si>
-  <si>
-    <t>O=C1OCC(F)O1</t>
-  </si>
-  <si>
     <t>Energy  retention at 5C discharge (25C)</t>
+  </si>
+  <si>
+    <t>Sum of EL wt%</t>
   </si>
 </sst>
 </file>
@@ -267,12 +237,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -299,10 +269,23 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -312,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -356,7 +339,6 @@
     <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -369,7 +351,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -380,6 +361,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -729,11 +722,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1950D208-EC04-4DB0-87B3-BAD1B195CB39}">
-  <dimension ref="A1:AJ374"/>
+  <dimension ref="A1:AK353"/>
   <sheetFormatPr defaultColWidth="9.08203125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="9.08203125" style="20"/>
-    <col min="3" max="3" width="14.9140625" style="20" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="9.08203125" style="19"/>
+    <col min="3" max="3" width="14.9140625" style="19" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.08203125" style="3"/>
     <col min="5" max="5" width="13.75" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.08203125" style="3"/>
@@ -741,12 +734,12 @@
     <col min="8" max="8" width="9.08203125" style="3"/>
     <col min="9" max="9" width="15" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="13" width="15" style="3" customWidth="1"/>
-    <col min="14" max="14" width="9.08203125" style="26"/>
-    <col min="15" max="15" width="13.4140625" style="26" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.08203125" style="26"/>
-    <col min="17" max="17" width="13.4140625" style="26" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.08203125" style="26"/>
-    <col min="19" max="19" width="13.4140625" style="26" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.08203125" style="24"/>
+    <col min="15" max="15" width="13.4140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.08203125" style="24"/>
+    <col min="17" max="17" width="13.4140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.08203125" style="24"/>
+    <col min="19" max="19" width="13.4140625" style="24" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9.4140625" style="4" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="13.75" style="4" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="9.4140625" style="4" bestFit="1" customWidth="1"/>
@@ -757,72 +750,75 @@
     <col min="27" max="27" width="13.75" style="4" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="9.4140625" style="4" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="13.75" style="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.75" style="4" customWidth="1"/>
-    <col min="31" max="31" width="13.75" style="22" customWidth="1"/>
+    <col min="30" max="31" width="13.75" style="4" customWidth="1"/>
     <col min="32" max="32" width="18.9140625" style="11" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="16.58203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.75" style="11" customWidth="1"/>
+    <col min="34" max="34" width="19.75" style="25" customWidth="1"/>
     <col min="35" max="35" width="19.08203125" style="12" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="26.9140625" style="10" customWidth="1"/>
-    <col min="37" max="16384" width="9.08203125" style="1"/>
+    <col min="37" max="37" width="12.9140625" style="1" customWidth="1"/>
+    <col min="38" max="16384" width="9.08203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A1" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="30" t="s">
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="31" t="s">
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="32"/>
+      <c r="T1" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="U1" s="33"/>
+      <c r="V1" s="33"/>
+      <c r="W1" s="33"/>
+      <c r="X1" s="33"/>
+      <c r="Y1" s="33"/>
+      <c r="Z1" s="33"/>
+      <c r="AA1" s="33"/>
+      <c r="AB1" s="33"/>
+      <c r="AC1" s="33"/>
+      <c r="AD1" s="21"/>
+      <c r="AE1" s="21"/>
+      <c r="AF1" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="31"/>
-      <c r="X1" s="31"/>
-      <c r="Y1" s="31"/>
-      <c r="Z1" s="31"/>
-      <c r="AA1" s="31"/>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="AG1" s="28"/>
-      <c r="AH1" s="28"/>
-      <c r="AI1" s="28"/>
-      <c r="AJ1" s="28"/>
-    </row>
-    <row r="2" spans="1:36" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
+      <c r="AG1" s="30"/>
+      <c r="AH1" s="30"/>
+      <c r="AI1" s="30"/>
+      <c r="AJ1" s="30"/>
+      <c r="AK1" s="27" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:37" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
       <c r="D2" s="5" t="s">
         <v>1</v>
       </c>
@@ -842,34 +838,34 @@
         <v>21</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="L2" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="N2" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="O2" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="P2" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q2" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="R2" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="S2" s="23" t="s">
         <v>34</v>
-      </c>
-      <c r="N2" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="O2" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="P2" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q2" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="R2" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="S2" s="25" t="s">
-        <v>35</v>
       </c>
       <c r="T2" s="6" t="s">
         <v>7</v>
@@ -902,10 +898,10 @@
         <v>16</v>
       </c>
       <c r="AD2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="AE2" s="8" t="s">
         <v>36</v>
-      </c>
-      <c r="AE2" s="8" t="s">
-        <v>37</v>
       </c>
       <c r="AF2" s="11" t="s">
         <v>26</v>
@@ -913,8 +909,8 @@
       <c r="AG2" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="AH2" s="11" t="s">
-        <v>50</v>
+      <c r="AH2" s="25" t="s">
+        <v>39</v>
       </c>
       <c r="AI2" s="11" t="s">
         <v>28</v>
@@ -922,2393 +918,2204 @@
       <c r="AJ2" s="11" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="A3" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" s="3">
-        <v>24.24</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G3" s="3">
-        <v>33.47</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I3" s="3">
-        <v>21.47</v>
-      </c>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
+      <c r="AK2" s="28"/>
+    </row>
+    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
       <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="O3" s="26">
-        <v>7.2</v>
-      </c>
-      <c r="P3" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q3" s="26">
-        <v>8.8699999999999992</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="U3" s="4">
-        <v>1.9</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="W3" s="4">
-        <v>1.9</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y3" s="4">
-        <v>0.95</v>
-      </c>
-      <c r="AE3" s="4"/>
-      <c r="AF3" s="11">
-        <v>1</v>
-      </c>
-      <c r="AG3" s="11">
-        <v>1</v>
-      </c>
-      <c r="AH3" s="11">
-        <v>1</v>
-      </c>
-      <c r="AI3" s="11">
-        <v>1</v>
-      </c>
-      <c r="AJ3" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="AE4" s="4"/>
+      <c r="M3" s="18"/>
+      <c r="AI3" s="11"/>
+      <c r="AJ3" s="11"/>
+    </row>
+    <row r="4" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J4" s="17"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="17"/>
+      <c r="M4" s="18"/>
       <c r="AI4" s="11"/>
       <c r="AJ4" s="11"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="AE5" s="4"/>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J5" s="17"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="18"/>
       <c r="AI5" s="11"/>
       <c r="AJ5" s="11"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="AE6" s="4"/>
+    <row r="6" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J6" s="17"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="18"/>
       <c r="AI6" s="11"/>
       <c r="AJ6" s="11"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="AE7" s="4"/>
+    <row r="7" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J7" s="17"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="18"/>
       <c r="AI7" s="11"/>
       <c r="AJ7" s="11"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="AE8" s="4"/>
+    <row r="8" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J8" s="17"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="18"/>
       <c r="AI8" s="11"/>
       <c r="AJ8" s="11"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="AE9" s="4"/>
+    <row r="9" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J9" s="17"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="17"/>
+      <c r="M9" s="18"/>
       <c r="AI9" s="11"/>
       <c r="AJ9" s="11"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="AE10" s="4"/>
+    <row r="10" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J10" s="17"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="18"/>
       <c r="AI10" s="11"/>
       <c r="AJ10" s="11"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="19"/>
-      <c r="AE11" s="4"/>
+    <row r="11" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J11" s="17"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="17"/>
+      <c r="M11" s="18"/>
       <c r="AI11" s="11"/>
       <c r="AJ11" s="11"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="AE12" s="4"/>
+    <row r="12" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J12" s="17"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="17"/>
+      <c r="M12" s="18"/>
       <c r="AI12" s="11"/>
       <c r="AJ12" s="11"/>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="19"/>
-      <c r="AE13" s="4"/>
+    <row r="13" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J13" s="17"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="17"/>
+      <c r="M13" s="18"/>
       <c r="AI13" s="11"/>
       <c r="AJ13" s="11"/>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="19"/>
-      <c r="AE14" s="4"/>
+    <row r="14" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J14" s="17"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="18"/>
       <c r="AI14" s="11"/>
       <c r="AJ14" s="11"/>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="19"/>
-      <c r="AE15" s="4"/>
+    <row r="15" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J15" s="17"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="18"/>
       <c r="AI15" s="11"/>
       <c r="AJ15" s="11"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="AE16" s="4"/>
+    <row r="16" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="J16" s="17"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="17"/>
+      <c r="M16" s="18"/>
       <c r="AI16" s="11"/>
       <c r="AJ16" s="11"/>
     </row>
     <row r="17" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="AE17" s="4"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="18"/>
       <c r="AI17" s="11"/>
       <c r="AJ17" s="11"/>
     </row>
     <row r="18" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="AE18" s="4"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="17"/>
+      <c r="M18" s="18"/>
       <c r="AI18" s="11"/>
       <c r="AJ18" s="11"/>
     </row>
     <row r="19" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="AE19" s="4"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="17"/>
+      <c r="M19" s="18"/>
       <c r="AI19" s="11"/>
       <c r="AJ19" s="11"/>
     </row>
     <row r="20" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="AE20" s="4"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="18"/>
       <c r="AI20" s="11"/>
       <c r="AJ20" s="11"/>
     </row>
     <row r="21" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="AE21" s="4"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="18"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="18"/>
       <c r="AI21" s="11"/>
       <c r="AJ21" s="11"/>
     </row>
     <row r="22" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="AE22" s="4"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="17"/>
+      <c r="M22" s="18"/>
       <c r="AI22" s="11"/>
       <c r="AJ22" s="11"/>
     </row>
     <row r="23" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="AE23" s="4"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="18"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="18"/>
       <c r="AI23" s="11"/>
       <c r="AJ23" s="11"/>
     </row>
     <row r="24" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J24" s="18"/>
-      <c r="K24" s="19"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="19"/>
-      <c r="AE24" s="4"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="18"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="18"/>
       <c r="AI24" s="11"/>
       <c r="AJ24" s="11"/>
     </row>
     <row r="25" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J25" s="18"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="19"/>
-      <c r="AE25" s="4"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="18"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="18"/>
       <c r="AI25" s="11"/>
       <c r="AJ25" s="11"/>
     </row>
     <row r="26" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J26" s="18"/>
-      <c r="K26" s="19"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="19"/>
-      <c r="AE26" s="4"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="18"/>
+      <c r="L26" s="17"/>
+      <c r="M26" s="18"/>
       <c r="AI26" s="11"/>
       <c r="AJ26" s="11"/>
     </row>
     <row r="27" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J27" s="18"/>
-      <c r="K27" s="19"/>
-      <c r="L27" s="18"/>
-      <c r="M27" s="19"/>
-      <c r="AE27" s="4"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="18"/>
       <c r="AI27" s="11"/>
       <c r="AJ27" s="11"/>
     </row>
     <row r="28" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J28" s="18"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="19"/>
-      <c r="AE28" s="4"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="18"/>
+      <c r="L28" s="17"/>
+      <c r="M28" s="18"/>
       <c r="AI28" s="11"/>
       <c r="AJ28" s="11"/>
     </row>
     <row r="29" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J29" s="18"/>
-      <c r="K29" s="19"/>
-      <c r="L29" s="18"/>
-      <c r="M29" s="19"/>
-      <c r="AE29" s="4"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="18"/>
+      <c r="L29" s="17"/>
+      <c r="M29" s="18"/>
       <c r="AI29" s="11"/>
       <c r="AJ29" s="11"/>
     </row>
     <row r="30" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J30" s="18"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="18"/>
-      <c r="M30" s="19"/>
-      <c r="AE30" s="4"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="18"/>
+      <c r="L30" s="17"/>
+      <c r="M30" s="18"/>
       <c r="AI30" s="11"/>
       <c r="AJ30" s="11"/>
     </row>
     <row r="31" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J31" s="18"/>
-      <c r="K31" s="19"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="19"/>
-      <c r="AE31" s="4"/>
+      <c r="J31" s="17"/>
+      <c r="K31" s="18"/>
+      <c r="L31" s="17"/>
+      <c r="M31" s="18"/>
       <c r="AI31" s="11"/>
       <c r="AJ31" s="11"/>
     </row>
     <row r="32" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J32" s="18"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="19"/>
-      <c r="AE32" s="4"/>
+      <c r="J32" s="17"/>
+      <c r="K32" s="17"/>
+      <c r="L32" s="17"/>
+      <c r="M32" s="17"/>
       <c r="AI32" s="11"/>
       <c r="AJ32" s="11"/>
     </row>
     <row r="33" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J33" s="18"/>
-      <c r="K33" s="19"/>
-      <c r="L33" s="18"/>
-      <c r="M33" s="19"/>
-      <c r="AE33" s="4"/>
+      <c r="J33" s="17"/>
+      <c r="K33" s="17"/>
+      <c r="L33" s="17"/>
+      <c r="M33" s="17"/>
       <c r="AI33" s="11"/>
       <c r="AJ33" s="11"/>
     </row>
     <row r="34" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J34" s="18"/>
-      <c r="K34" s="19"/>
-      <c r="L34" s="18"/>
-      <c r="M34" s="19"/>
-      <c r="AE34" s="4"/>
+      <c r="J34" s="17"/>
+      <c r="K34" s="17"/>
+      <c r="L34" s="17"/>
+      <c r="M34" s="17"/>
       <c r="AI34" s="11"/>
       <c r="AJ34" s="11"/>
     </row>
     <row r="35" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J35" s="18"/>
-      <c r="K35" s="19"/>
-      <c r="L35" s="18"/>
-      <c r="M35" s="19"/>
-      <c r="AE35" s="4"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+      <c r="L35" s="17"/>
+      <c r="M35" s="17"/>
       <c r="AI35" s="11"/>
       <c r="AJ35" s="11"/>
     </row>
     <row r="36" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J36" s="18"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="18"/>
-      <c r="M36" s="19"/>
-      <c r="AE36" s="4"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
       <c r="AI36" s="11"/>
       <c r="AJ36" s="11"/>
     </row>
     <row r="37" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J37" s="18"/>
-      <c r="K37" s="19"/>
-      <c r="L37" s="18"/>
-      <c r="M37" s="19"/>
-      <c r="AE37" s="4"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17"/>
+      <c r="M37" s="17"/>
       <c r="AI37" s="11"/>
       <c r="AJ37" s="11"/>
     </row>
     <row r="38" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J38" s="18"/>
-      <c r="K38" s="19"/>
-      <c r="L38" s="18"/>
-      <c r="M38" s="19"/>
-      <c r="AE38" s="4"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
       <c r="AI38" s="11"/>
       <c r="AJ38" s="11"/>
     </row>
     <row r="39" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J39" s="18"/>
-      <c r="K39" s="19"/>
-      <c r="L39" s="18"/>
-      <c r="M39" s="19"/>
-      <c r="AE39" s="4"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="17"/>
+      <c r="M39" s="17"/>
       <c r="AI39" s="11"/>
       <c r="AJ39" s="11"/>
     </row>
     <row r="40" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J40" s="18"/>
-      <c r="K40" s="19"/>
-      <c r="L40" s="18"/>
-      <c r="M40" s="19"/>
-      <c r="AE40" s="4"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
+      <c r="L40" s="17"/>
+      <c r="M40" s="17"/>
       <c r="AI40" s="11"/>
       <c r="AJ40" s="11"/>
     </row>
     <row r="41" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J41" s="18"/>
-      <c r="K41" s="19"/>
-      <c r="L41" s="18"/>
-      <c r="M41" s="19"/>
-      <c r="AE41" s="4"/>
+      <c r="J41" s="17"/>
+      <c r="K41" s="17"/>
+      <c r="L41" s="17"/>
+      <c r="M41" s="17"/>
       <c r="AI41" s="11"/>
       <c r="AJ41" s="11"/>
     </row>
     <row r="42" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J42" s="18"/>
-      <c r="K42" s="19"/>
-      <c r="L42" s="18"/>
-      <c r="M42" s="19"/>
-      <c r="AE42" s="4"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="17"/>
+      <c r="L42" s="17"/>
+      <c r="M42" s="17"/>
       <c r="AI42" s="11"/>
       <c r="AJ42" s="11"/>
     </row>
     <row r="43" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J43" s="18"/>
-      <c r="K43" s="19"/>
-      <c r="L43" s="18"/>
-      <c r="M43" s="19"/>
-      <c r="AE43" s="4"/>
-      <c r="AI43" s="11"/>
-      <c r="AJ43" s="11"/>
+      <c r="AF43" s="9"/>
+      <c r="AG43" s="9"/>
+      <c r="AH43" s="15"/>
+      <c r="AI43" s="10"/>
     </row>
     <row r="44" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J44" s="18"/>
-      <c r="K44" s="19"/>
-      <c r="L44" s="18"/>
-      <c r="M44" s="19"/>
-      <c r="AE44" s="4"/>
-      <c r="AI44" s="11"/>
-      <c r="AJ44" s="11"/>
+      <c r="AF44" s="9"/>
+      <c r="AG44" s="9"/>
+      <c r="AH44" s="15"/>
+      <c r="AI44" s="10"/>
     </row>
     <row r="45" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J45" s="18"/>
-      <c r="K45" s="19"/>
-      <c r="L45" s="18"/>
-      <c r="M45" s="19"/>
-      <c r="AE45" s="4"/>
-      <c r="AI45" s="11"/>
-      <c r="AJ45" s="11"/>
+      <c r="AF45" s="9"/>
+      <c r="AG45" s="9"/>
+      <c r="AH45" s="15"/>
+      <c r="AI45" s="10"/>
     </row>
     <row r="46" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J46" s="18"/>
-      <c r="K46" s="19"/>
-      <c r="L46" s="18"/>
-      <c r="M46" s="19"/>
-      <c r="AE46" s="4"/>
-      <c r="AI46" s="11"/>
-      <c r="AJ46" s="11"/>
+      <c r="AF46" s="9"/>
+      <c r="AG46" s="9"/>
+      <c r="AH46" s="15"/>
+      <c r="AI46" s="10"/>
     </row>
     <row r="47" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J47" s="18"/>
-      <c r="K47" s="19"/>
-      <c r="L47" s="18"/>
-      <c r="M47" s="19"/>
-      <c r="AE47" s="4"/>
-      <c r="AI47" s="11"/>
-      <c r="AJ47" s="11"/>
+      <c r="AF47" s="9"/>
+      <c r="AG47" s="9"/>
+      <c r="AH47" s="15"/>
+      <c r="AI47" s="10"/>
     </row>
     <row r="48" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J48" s="18"/>
-      <c r="K48" s="19"/>
-      <c r="L48" s="18"/>
-      <c r="M48" s="19"/>
-      <c r="AE48" s="4"/>
-      <c r="AI48" s="11"/>
-      <c r="AJ48" s="11"/>
-    </row>
-    <row r="49" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J49" s="18"/>
-      <c r="K49" s="19"/>
-      <c r="L49" s="18"/>
-      <c r="M49" s="19"/>
-      <c r="AE49" s="4"/>
-      <c r="AI49" s="11"/>
-      <c r="AJ49" s="11"/>
-    </row>
-    <row r="50" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J50" s="18"/>
-      <c r="K50" s="19"/>
-      <c r="L50" s="18"/>
-      <c r="M50" s="19"/>
-      <c r="AE50" s="4"/>
-      <c r="AI50" s="11"/>
-      <c r="AJ50" s="11"/>
-    </row>
-    <row r="51" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J51" s="18"/>
-      <c r="K51" s="19"/>
-      <c r="L51" s="18"/>
-      <c r="M51" s="19"/>
-      <c r="AE51" s="4"/>
-      <c r="AI51" s="11"/>
-      <c r="AJ51" s="11"/>
-    </row>
-    <row r="52" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J52" s="18"/>
-      <c r="K52" s="19"/>
-      <c r="L52" s="18"/>
-      <c r="M52" s="19"/>
-      <c r="AE52" s="4"/>
-      <c r="AI52" s="11"/>
-      <c r="AJ52" s="11"/>
-    </row>
-    <row r="53" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J53" s="18"/>
-      <c r="K53" s="18"/>
-      <c r="L53" s="18"/>
-      <c r="M53" s="18"/>
-      <c r="AE53" s="4"/>
-      <c r="AI53" s="11"/>
-      <c r="AJ53" s="11"/>
-    </row>
-    <row r="54" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J54" s="18"/>
-      <c r="K54" s="18"/>
-      <c r="L54" s="18"/>
-      <c r="M54" s="18"/>
-      <c r="AE54" s="4"/>
-      <c r="AI54" s="11"/>
-      <c r="AJ54" s="11"/>
-    </row>
-    <row r="55" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J55" s="18"/>
-      <c r="K55" s="18"/>
-      <c r="L55" s="18"/>
-      <c r="M55" s="18"/>
-      <c r="AE55" s="4"/>
-      <c r="AI55" s="11"/>
-      <c r="AJ55" s="11"/>
-    </row>
-    <row r="56" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J56" s="18"/>
-      <c r="K56" s="18"/>
-      <c r="L56" s="18"/>
-      <c r="M56" s="18"/>
-      <c r="AE56" s="4"/>
-      <c r="AI56" s="11"/>
-      <c r="AJ56" s="11"/>
-    </row>
-    <row r="57" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J57" s="18"/>
-      <c r="K57" s="18"/>
-      <c r="L57" s="18"/>
-      <c r="M57" s="18"/>
-      <c r="AE57" s="4"/>
-      <c r="AI57" s="11"/>
-      <c r="AJ57" s="11"/>
-    </row>
-    <row r="58" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J58" s="18"/>
-      <c r="K58" s="18"/>
-      <c r="L58" s="18"/>
-      <c r="M58" s="18"/>
-      <c r="AE58" s="4"/>
-      <c r="AI58" s="11"/>
-      <c r="AJ58" s="11"/>
-    </row>
-    <row r="59" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J59" s="18"/>
-      <c r="K59" s="18"/>
-      <c r="L59" s="18"/>
-      <c r="M59" s="18"/>
-      <c r="AE59" s="4"/>
-      <c r="AI59" s="11"/>
-      <c r="AJ59" s="11"/>
-    </row>
-    <row r="60" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J60" s="18"/>
-      <c r="K60" s="18"/>
-      <c r="L60" s="18"/>
-      <c r="M60" s="18"/>
-      <c r="AE60" s="4"/>
-      <c r="AI60" s="11"/>
-      <c r="AJ60" s="11"/>
-    </row>
-    <row r="61" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J61" s="18"/>
-      <c r="K61" s="18"/>
-      <c r="L61" s="18"/>
-      <c r="M61" s="18"/>
-      <c r="AE61" s="4"/>
-      <c r="AI61" s="11"/>
-      <c r="AJ61" s="11"/>
-    </row>
-    <row r="62" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J62" s="18"/>
-      <c r="K62" s="18"/>
-      <c r="L62" s="18"/>
-      <c r="M62" s="18"/>
-      <c r="AE62" s="4"/>
-      <c r="AI62" s="11"/>
-      <c r="AJ62" s="11"/>
-    </row>
-    <row r="63" spans="10:36" x14ac:dyDescent="0.3">
-      <c r="J63" s="18"/>
-      <c r="K63" s="18"/>
-      <c r="L63" s="18"/>
-      <c r="M63" s="18"/>
-      <c r="AE63" s="4"/>
-      <c r="AI63" s="11"/>
-      <c r="AJ63" s="11"/>
-    </row>
-    <row r="64" spans="10:36" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="65" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="66" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="67" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="68" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="69" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="70" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="71" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="72" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="73" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="74" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="75" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="76" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="81" spans="32:35" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="82" spans="32:35" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="83" spans="32:35" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="84" spans="32:35" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="85" spans="32:35" customFormat="1" x14ac:dyDescent="0.3"/>
+      <c r="AF48" s="9"/>
+      <c r="AG48" s="9"/>
+      <c r="AH48" s="15"/>
+      <c r="AI48" s="10"/>
+    </row>
+    <row r="49" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF49" s="9"/>
+      <c r="AG49" s="9"/>
+      <c r="AH49" s="15"/>
+      <c r="AI49" s="10"/>
+    </row>
+    <row r="50" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF50" s="9"/>
+      <c r="AG50" s="9"/>
+      <c r="AH50" s="15"/>
+      <c r="AI50" s="10"/>
+    </row>
+    <row r="51" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF51" s="9"/>
+      <c r="AG51" s="9"/>
+      <c r="AH51" s="15"/>
+      <c r="AI51" s="10"/>
+    </row>
+    <row r="52" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF52" s="9"/>
+      <c r="AG52" s="9"/>
+      <c r="AH52" s="15"/>
+      <c r="AI52" s="10"/>
+    </row>
+    <row r="53" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF53" s="9"/>
+      <c r="AG53" s="9"/>
+      <c r="AH53" s="15"/>
+      <c r="AI53" s="10"/>
+    </row>
+    <row r="54" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF54" s="9"/>
+      <c r="AG54" s="9"/>
+      <c r="AH54" s="15"/>
+      <c r="AI54" s="10"/>
+    </row>
+    <row r="55" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF55" s="9"/>
+      <c r="AG55" s="9"/>
+      <c r="AH55" s="15"/>
+      <c r="AI55" s="10"/>
+    </row>
+    <row r="56" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF56" s="9"/>
+      <c r="AG56" s="9"/>
+      <c r="AH56" s="15"/>
+      <c r="AI56" s="10"/>
+    </row>
+    <row r="57" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF57" s="9"/>
+      <c r="AG57" s="9"/>
+      <c r="AH57" s="15"/>
+      <c r="AI57" s="10"/>
+    </row>
+    <row r="58" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF58" s="9"/>
+      <c r="AG58" s="9"/>
+      <c r="AH58" s="15"/>
+      <c r="AI58" s="10"/>
+    </row>
+    <row r="59" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF59" s="9"/>
+      <c r="AG59" s="9"/>
+      <c r="AH59" s="15"/>
+      <c r="AI59" s="10"/>
+    </row>
+    <row r="60" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF60" s="9"/>
+      <c r="AG60" s="9"/>
+      <c r="AH60" s="15"/>
+      <c r="AI60" s="10"/>
+    </row>
+    <row r="61" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF61" s="9"/>
+      <c r="AG61" s="9"/>
+      <c r="AH61" s="15"/>
+      <c r="AI61" s="10"/>
+    </row>
+    <row r="62" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF62" s="9"/>
+      <c r="AG62" s="9"/>
+      <c r="AH62" s="15"/>
+      <c r="AI62" s="10"/>
+    </row>
+    <row r="63" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF63" s="9"/>
+      <c r="AG63" s="9"/>
+      <c r="AH63" s="15"/>
+      <c r="AI63" s="10"/>
+    </row>
+    <row r="64" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF64" s="9"/>
+      <c r="AG64" s="9"/>
+      <c r="AH64" s="15"/>
+      <c r="AI64" s="10"/>
+    </row>
+    <row r="65" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF65" s="9"/>
+      <c r="AG65" s="9"/>
+      <c r="AH65" s="15"/>
+      <c r="AI65" s="10"/>
+    </row>
+    <row r="66" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF66" s="9"/>
+      <c r="AG66" s="9"/>
+      <c r="AH66" s="15"/>
+      <c r="AI66" s="10"/>
+    </row>
+    <row r="67" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF67" s="9"/>
+      <c r="AG67" s="9"/>
+      <c r="AH67" s="15"/>
+      <c r="AI67" s="10"/>
+    </row>
+    <row r="68" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF68" s="9"/>
+      <c r="AG68" s="9"/>
+      <c r="AH68" s="15"/>
+      <c r="AI68" s="10"/>
+    </row>
+    <row r="69" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF69" s="9"/>
+      <c r="AG69" s="9"/>
+      <c r="AH69" s="15"/>
+      <c r="AI69" s="10"/>
+    </row>
+    <row r="70" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF70" s="9"/>
+      <c r="AG70" s="9"/>
+      <c r="AH70" s="15"/>
+      <c r="AI70" s="10"/>
+    </row>
+    <row r="71" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF71" s="9"/>
+      <c r="AG71" s="9"/>
+      <c r="AH71" s="15"/>
+      <c r="AI71" s="10"/>
+    </row>
+    <row r="72" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF72" s="9"/>
+      <c r="AG72" s="9"/>
+      <c r="AH72" s="15"/>
+      <c r="AI72" s="10"/>
+    </row>
+    <row r="73" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF73" s="9"/>
+      <c r="AG73" s="9"/>
+      <c r="AH73" s="15"/>
+      <c r="AI73" s="10"/>
+    </row>
+    <row r="74" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF74" s="9"/>
+      <c r="AG74" s="9"/>
+      <c r="AH74" s="15"/>
+      <c r="AI74" s="10"/>
+    </row>
+    <row r="75" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF75" s="9"/>
+      <c r="AG75" s="9"/>
+      <c r="AH75" s="15"/>
+      <c r="AI75" s="10"/>
+    </row>
+    <row r="76" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF76" s="9"/>
+      <c r="AG76" s="9"/>
+      <c r="AH76" s="15"/>
+      <c r="AI76" s="10"/>
+    </row>
+    <row r="77" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF77" s="9"/>
+      <c r="AG77" s="9"/>
+      <c r="AH77" s="15"/>
+      <c r="AI77" s="10"/>
+    </row>
+    <row r="78" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF78" s="9"/>
+      <c r="AG78" s="9"/>
+      <c r="AH78" s="15"/>
+      <c r="AI78" s="10"/>
+    </row>
+    <row r="79" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF79" s="9"/>
+      <c r="AG79" s="9"/>
+      <c r="AH79" s="15"/>
+      <c r="AI79" s="10"/>
+    </row>
+    <row r="80" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF80" s="9"/>
+      <c r="AG80" s="9"/>
+      <c r="AH80" s="15"/>
+      <c r="AI80" s="10"/>
+    </row>
+    <row r="81" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF81" s="9"/>
+      <c r="AG81" s="9"/>
+      <c r="AH81" s="15"/>
+      <c r="AI81" s="10"/>
+    </row>
+    <row r="82" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF82" s="9"/>
+      <c r="AG82" s="9"/>
+      <c r="AH82" s="15"/>
+      <c r="AI82" s="10"/>
+    </row>
+    <row r="83" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF83" s="9"/>
+      <c r="AG83" s="9"/>
+      <c r="AH83" s="15"/>
+      <c r="AI83" s="10"/>
+    </row>
+    <row r="84" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF84" s="9"/>
+      <c r="AG84" s="9"/>
+      <c r="AH84" s="15"/>
+      <c r="AI84" s="10"/>
+    </row>
+    <row r="85" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AF85" s="9"/>
+      <c r="AG85" s="9"/>
+      <c r="AH85" s="15"/>
+      <c r="AI85" s="10"/>
+    </row>
     <row r="86" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF86" s="9"/>
       <c r="AG86" s="9"/>
-      <c r="AH86" s="9"/>
+      <c r="AH86" s="15"/>
       <c r="AI86" s="10"/>
     </row>
     <row r="87" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF87" s="9"/>
       <c r="AG87" s="9"/>
-      <c r="AH87" s="9"/>
+      <c r="AH87" s="15"/>
       <c r="AI87" s="10"/>
     </row>
     <row r="88" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF88" s="9"/>
       <c r="AG88" s="9"/>
-      <c r="AH88" s="9"/>
+      <c r="AH88" s="15"/>
       <c r="AI88" s="10"/>
     </row>
     <row r="89" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF89" s="9"/>
       <c r="AG89" s="9"/>
-      <c r="AH89" s="9"/>
+      <c r="AH89" s="15"/>
       <c r="AI89" s="10"/>
     </row>
     <row r="90" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF90" s="9"/>
       <c r="AG90" s="9"/>
-      <c r="AH90" s="9"/>
+      <c r="AH90" s="15"/>
       <c r="AI90" s="10"/>
     </row>
     <row r="91" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF91" s="9"/>
       <c r="AG91" s="9"/>
-      <c r="AH91" s="9"/>
+      <c r="AH91" s="15"/>
       <c r="AI91" s="10"/>
     </row>
     <row r="92" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF92" s="9"/>
       <c r="AG92" s="9"/>
-      <c r="AH92" s="9"/>
+      <c r="AH92" s="15"/>
       <c r="AI92" s="10"/>
     </row>
     <row r="93" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF93" s="9"/>
       <c r="AG93" s="9"/>
-      <c r="AH93" s="9"/>
+      <c r="AH93" s="15"/>
       <c r="AI93" s="10"/>
     </row>
     <row r="94" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF94" s="9"/>
       <c r="AG94" s="9"/>
-      <c r="AH94" s="9"/>
+      <c r="AH94" s="15"/>
       <c r="AI94" s="10"/>
     </row>
     <row r="95" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF95" s="9"/>
       <c r="AG95" s="9"/>
-      <c r="AH95" s="9"/>
+      <c r="AH95" s="15"/>
       <c r="AI95" s="10"/>
     </row>
     <row r="96" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF96" s="9"/>
       <c r="AG96" s="9"/>
-      <c r="AH96" s="9"/>
+      <c r="AH96" s="15"/>
       <c r="AI96" s="10"/>
     </row>
     <row r="97" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF97" s="9"/>
       <c r="AG97" s="9"/>
-      <c r="AH97" s="9"/>
+      <c r="AH97" s="15"/>
       <c r="AI97" s="10"/>
     </row>
     <row r="98" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF98" s="9"/>
       <c r="AG98" s="9"/>
-      <c r="AH98" s="9"/>
+      <c r="AH98" s="15"/>
       <c r="AI98" s="10"/>
     </row>
     <row r="99" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF99" s="9"/>
       <c r="AG99" s="9"/>
-      <c r="AH99" s="9"/>
+      <c r="AH99" s="15"/>
       <c r="AI99" s="10"/>
     </row>
     <row r="100" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF100" s="9"/>
       <c r="AG100" s="9"/>
-      <c r="AH100" s="9"/>
+      <c r="AH100" s="15"/>
       <c r="AI100" s="10"/>
     </row>
     <row r="101" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF101" s="9"/>
       <c r="AG101" s="9"/>
-      <c r="AH101" s="9"/>
+      <c r="AH101" s="15"/>
       <c r="AI101" s="10"/>
     </row>
     <row r="102" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF102" s="9"/>
       <c r="AG102" s="9"/>
-      <c r="AH102" s="9"/>
+      <c r="AH102" s="15"/>
       <c r="AI102" s="10"/>
     </row>
     <row r="103" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF103" s="9"/>
       <c r="AG103" s="9"/>
-      <c r="AH103" s="9"/>
+      <c r="AH103" s="15"/>
       <c r="AI103" s="10"/>
     </row>
     <row r="104" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF104" s="9"/>
       <c r="AG104" s="9"/>
-      <c r="AH104" s="9"/>
+      <c r="AH104" s="15"/>
       <c r="AI104" s="10"/>
     </row>
     <row r="105" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF105" s="9"/>
       <c r="AG105" s="9"/>
-      <c r="AH105" s="9"/>
+      <c r="AH105" s="15"/>
       <c r="AI105" s="10"/>
     </row>
     <row r="106" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF106" s="9"/>
       <c r="AG106" s="9"/>
-      <c r="AH106" s="9"/>
+      <c r="AH106" s="15"/>
       <c r="AI106" s="10"/>
     </row>
     <row r="107" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF107" s="9"/>
       <c r="AG107" s="9"/>
-      <c r="AH107" s="9"/>
+      <c r="AH107" s="15"/>
       <c r="AI107" s="10"/>
     </row>
     <row r="108" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF108" s="9"/>
       <c r="AG108" s="9"/>
-      <c r="AH108" s="9"/>
+      <c r="AH108" s="15"/>
       <c r="AI108" s="10"/>
     </row>
     <row r="109" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF109" s="9"/>
       <c r="AG109" s="9"/>
-      <c r="AH109" s="9"/>
+      <c r="AH109" s="15"/>
       <c r="AI109" s="10"/>
     </row>
     <row r="110" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF110" s="9"/>
       <c r="AG110" s="9"/>
-      <c r="AH110" s="9"/>
+      <c r="AH110" s="15"/>
       <c r="AI110" s="10"/>
     </row>
     <row r="111" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF111" s="9"/>
       <c r="AG111" s="9"/>
-      <c r="AH111" s="9"/>
+      <c r="AH111" s="15"/>
       <c r="AI111" s="10"/>
     </row>
     <row r="112" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF112" s="9"/>
       <c r="AG112" s="9"/>
-      <c r="AH112" s="9"/>
+      <c r="AH112" s="15"/>
       <c r="AI112" s="10"/>
     </row>
     <row r="113" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF113" s="9"/>
       <c r="AG113" s="9"/>
-      <c r="AH113" s="9"/>
+      <c r="AH113" s="15"/>
       <c r="AI113" s="10"/>
     </row>
     <row r="114" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF114" s="9"/>
       <c r="AG114" s="9"/>
-      <c r="AH114" s="9"/>
+      <c r="AH114" s="15"/>
       <c r="AI114" s="10"/>
     </row>
     <row r="115" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF115" s="9"/>
       <c r="AG115" s="9"/>
-      <c r="AH115" s="9"/>
+      <c r="AH115" s="15"/>
       <c r="AI115" s="10"/>
     </row>
     <row r="116" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF116" s="9"/>
       <c r="AG116" s="9"/>
-      <c r="AH116" s="9"/>
+      <c r="AH116" s="15"/>
       <c r="AI116" s="10"/>
     </row>
     <row r="117" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF117" s="9"/>
       <c r="AG117" s="9"/>
-      <c r="AH117" s="9"/>
+      <c r="AH117" s="15"/>
       <c r="AI117" s="10"/>
     </row>
     <row r="118" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF118" s="9"/>
       <c r="AG118" s="9"/>
-      <c r="AH118" s="9"/>
+      <c r="AH118" s="15"/>
       <c r="AI118" s="10"/>
     </row>
     <row r="119" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF119" s="9"/>
       <c r="AG119" s="9"/>
-      <c r="AH119" s="9"/>
+      <c r="AH119" s="15"/>
       <c r="AI119" s="10"/>
     </row>
     <row r="120" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF120" s="9"/>
       <c r="AG120" s="9"/>
-      <c r="AH120" s="9"/>
+      <c r="AH120" s="15"/>
       <c r="AI120" s="10"/>
     </row>
     <row r="121" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF121" s="9"/>
       <c r="AG121" s="9"/>
-      <c r="AH121" s="9"/>
+      <c r="AH121" s="15"/>
       <c r="AI121" s="10"/>
     </row>
     <row r="122" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF122" s="9"/>
       <c r="AG122" s="9"/>
-      <c r="AH122" s="9"/>
+      <c r="AH122" s="15"/>
       <c r="AI122" s="10"/>
     </row>
     <row r="123" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF123" s="9"/>
       <c r="AG123" s="9"/>
-      <c r="AH123" s="9"/>
+      <c r="AH123" s="15"/>
       <c r="AI123" s="10"/>
     </row>
     <row r="124" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF124" s="9"/>
       <c r="AG124" s="9"/>
-      <c r="AH124" s="9"/>
+      <c r="AH124" s="15"/>
       <c r="AI124" s="10"/>
     </row>
     <row r="125" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF125" s="9"/>
       <c r="AG125" s="9"/>
-      <c r="AH125" s="9"/>
+      <c r="AH125" s="15"/>
       <c r="AI125" s="10"/>
     </row>
     <row r="126" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF126" s="9"/>
       <c r="AG126" s="9"/>
-      <c r="AH126" s="9"/>
+      <c r="AH126" s="15"/>
       <c r="AI126" s="10"/>
     </row>
     <row r="127" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF127" s="9"/>
       <c r="AG127" s="9"/>
-      <c r="AH127" s="9"/>
+      <c r="AH127" s="15"/>
       <c r="AI127" s="10"/>
     </row>
     <row r="128" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF128" s="9"/>
       <c r="AG128" s="9"/>
-      <c r="AH128" s="9"/>
+      <c r="AH128" s="15"/>
       <c r="AI128" s="10"/>
     </row>
-    <row r="129" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="129" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF129" s="9"/>
       <c r="AG129" s="9"/>
-      <c r="AH129" s="9"/>
+      <c r="AH129" s="15"/>
       <c r="AI129" s="10"/>
     </row>
-    <row r="130" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="130" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF130" s="9"/>
       <c r="AG130" s="9"/>
-      <c r="AH130" s="9"/>
+      <c r="AH130" s="15"/>
       <c r="AI130" s="10"/>
     </row>
-    <row r="131" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="131" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF131" s="9"/>
       <c r="AG131" s="9"/>
-      <c r="AH131" s="9"/>
+      <c r="AH131" s="15"/>
       <c r="AI131" s="10"/>
     </row>
-    <row r="132" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="132" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF132" s="9"/>
       <c r="AG132" s="9"/>
-      <c r="AH132" s="9"/>
+      <c r="AH132" s="15"/>
       <c r="AI132" s="10"/>
     </row>
-    <row r="133" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="133" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF133" s="9"/>
       <c r="AG133" s="9"/>
-      <c r="AH133" s="9"/>
+      <c r="AH133" s="15"/>
       <c r="AI133" s="10"/>
     </row>
-    <row r="134" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="134" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF134" s="9"/>
       <c r="AG134" s="9"/>
-      <c r="AH134" s="9"/>
+      <c r="AH134" s="15"/>
       <c r="AI134" s="10"/>
     </row>
-    <row r="135" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="135" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF135" s="9"/>
       <c r="AG135" s="9"/>
-      <c r="AH135" s="9"/>
+      <c r="AH135" s="15"/>
       <c r="AI135" s="10"/>
     </row>
-    <row r="136" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="136" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF136" s="9"/>
       <c r="AG136" s="9"/>
-      <c r="AH136" s="9"/>
+      <c r="AH136" s="15"/>
       <c r="AI136" s="10"/>
     </row>
-    <row r="137" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="137" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF137" s="9"/>
       <c r="AG137" s="9"/>
-      <c r="AH137" s="9"/>
+      <c r="AH137" s="15"/>
       <c r="AI137" s="10"/>
     </row>
-    <row r="138" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="138" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF138" s="9"/>
       <c r="AG138" s="9"/>
-      <c r="AH138" s="9"/>
+      <c r="AH138" s="15"/>
       <c r="AI138" s="10"/>
     </row>
-    <row r="139" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="139" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF139" s="9"/>
       <c r="AG139" s="9"/>
-      <c r="AH139" s="9"/>
+      <c r="AH139" s="15"/>
       <c r="AI139" s="10"/>
     </row>
-    <row r="140" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="140" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF140" s="9"/>
       <c r="AG140" s="9"/>
-      <c r="AH140" s="9"/>
+      <c r="AH140" s="15"/>
       <c r="AI140" s="10"/>
     </row>
-    <row r="141" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="141" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF141" s="9"/>
       <c r="AG141" s="9"/>
-      <c r="AH141" s="9"/>
+      <c r="AH141" s="15"/>
       <c r="AI141" s="10"/>
     </row>
-    <row r="142" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="142" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF142" s="9"/>
       <c r="AG142" s="9"/>
-      <c r="AH142" s="9"/>
+      <c r="AH142" s="15"/>
       <c r="AI142" s="10"/>
     </row>
-    <row r="143" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="143" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF143" s="9"/>
       <c r="AG143" s="9"/>
-      <c r="AH143" s="9"/>
+      <c r="AH143" s="15"/>
       <c r="AI143" s="10"/>
     </row>
-    <row r="144" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="144" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF144" s="9"/>
-      <c r="AG144" s="9"/>
-      <c r="AH144" s="9"/>
-      <c r="AI144" s="10"/>
-    </row>
-    <row r="145" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ144" s="12"/>
+    </row>
+    <row r="145" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF145" s="9"/>
-      <c r="AG145" s="9"/>
-      <c r="AH145" s="9"/>
-      <c r="AI145" s="10"/>
-    </row>
-    <row r="146" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ145" s="12"/>
+    </row>
+    <row r="146" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF146" s="9"/>
-      <c r="AG146" s="9"/>
-      <c r="AH146" s="9"/>
-      <c r="AI146" s="10"/>
-    </row>
-    <row r="147" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ146" s="12"/>
+    </row>
+    <row r="147" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF147" s="9"/>
-      <c r="AG147" s="9"/>
-      <c r="AH147" s="9"/>
-      <c r="AI147" s="10"/>
-    </row>
-    <row r="148" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ147" s="12"/>
+    </row>
+    <row r="148" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF148" s="9"/>
-      <c r="AG148" s="9"/>
-      <c r="AH148" s="9"/>
-      <c r="AI148" s="10"/>
-    </row>
-    <row r="149" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ148" s="12"/>
+    </row>
+    <row r="149" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF149" s="9"/>
-      <c r="AG149" s="9"/>
-      <c r="AH149" s="9"/>
-      <c r="AI149" s="10"/>
-    </row>
-    <row r="150" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ149" s="12"/>
+    </row>
+    <row r="150" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF150" s="9"/>
-      <c r="AG150" s="9"/>
-      <c r="AH150" s="9"/>
-      <c r="AI150" s="10"/>
-    </row>
-    <row r="151" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ150" s="12"/>
+    </row>
+    <row r="151" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF151" s="9"/>
-      <c r="AG151" s="9"/>
-      <c r="AH151" s="9"/>
-      <c r="AI151" s="10"/>
-    </row>
-    <row r="152" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ151" s="12"/>
+    </row>
+    <row r="152" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF152" s="9"/>
       <c r="AG152" s="9"/>
-      <c r="AH152" s="9"/>
+      <c r="AH152" s="15"/>
       <c r="AI152" s="10"/>
     </row>
-    <row r="153" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="153" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF153" s="9"/>
       <c r="AG153" s="9"/>
-      <c r="AH153" s="9"/>
+      <c r="AH153" s="15"/>
       <c r="AI153" s="10"/>
     </row>
-    <row r="154" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="154" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF154" s="9"/>
       <c r="AG154" s="9"/>
-      <c r="AH154" s="9"/>
+      <c r="AH154" s="15"/>
       <c r="AI154" s="10"/>
     </row>
-    <row r="155" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="155" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF155" s="9"/>
-      <c r="AG155" s="9"/>
-      <c r="AH155" s="9"/>
-      <c r="AI155" s="10"/>
-    </row>
-    <row r="156" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ155" s="12"/>
+    </row>
+    <row r="156" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF156" s="9"/>
-      <c r="AG156" s="9"/>
-      <c r="AH156" s="9"/>
-      <c r="AI156" s="10"/>
-    </row>
-    <row r="157" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ156" s="12"/>
+    </row>
+    <row r="157" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF157" s="9"/>
-      <c r="AG157" s="9"/>
-      <c r="AH157" s="9"/>
-      <c r="AI157" s="10"/>
-    </row>
-    <row r="158" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ157" s="12"/>
+    </row>
+    <row r="158" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF158" s="9"/>
-      <c r="AG158" s="9"/>
-      <c r="AH158" s="9"/>
-      <c r="AI158" s="10"/>
-    </row>
-    <row r="159" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ158" s="12"/>
+    </row>
+    <row r="159" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF159" s="9"/>
-      <c r="AG159" s="9"/>
-      <c r="AH159" s="9"/>
-      <c r="AI159" s="10"/>
-    </row>
-    <row r="160" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ159" s="12"/>
+    </row>
+    <row r="160" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF160" s="9"/>
-      <c r="AG160" s="9"/>
-      <c r="AH160" s="9"/>
-      <c r="AI160" s="10"/>
+      <c r="AJ160" s="12"/>
     </row>
     <row r="161" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF161" s="9"/>
-      <c r="AG161" s="9"/>
-      <c r="AH161" s="9"/>
-      <c r="AI161" s="10"/>
+      <c r="AJ161" s="12"/>
     </row>
     <row r="162" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF162" s="9"/>
-      <c r="AG162" s="9"/>
-      <c r="AH162" s="9"/>
-      <c r="AI162" s="10"/>
+      <c r="AJ162" s="12"/>
     </row>
     <row r="163" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF163" s="9"/>
-      <c r="AG163" s="9"/>
-      <c r="AH163" s="9"/>
-      <c r="AI163" s="10"/>
+      <c r="AJ163" s="12"/>
     </row>
     <row r="164" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF164" s="9"/>
       <c r="AG164" s="9"/>
-      <c r="AH164" s="9"/>
+      <c r="AH164" s="15"/>
       <c r="AI164" s="10"/>
     </row>
     <row r="165" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF165" s="9"/>
-      <c r="AJ165" s="12"/>
+      <c r="AG165" s="9"/>
+      <c r="AH165" s="15"/>
+      <c r="AI165" s="10"/>
     </row>
     <row r="166" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF166" s="9"/>
-      <c r="AJ166" s="12"/>
+      <c r="AG166" s="9"/>
+      <c r="AH166" s="15"/>
+      <c r="AI166" s="10"/>
     </row>
     <row r="167" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF167" s="9"/>
-      <c r="AJ167" s="12"/>
+      <c r="AG167" s="9"/>
+      <c r="AH167" s="15"/>
+      <c r="AI167" s="10"/>
     </row>
     <row r="168" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF168" s="9"/>
-      <c r="AJ168" s="12"/>
+      <c r="AG168" s="9"/>
+      <c r="AH168" s="15"/>
+      <c r="AI168" s="10"/>
     </row>
     <row r="169" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF169" s="9"/>
-      <c r="AJ169" s="12"/>
+      <c r="AG169" s="9"/>
+      <c r="AH169" s="15"/>
+      <c r="AI169" s="10"/>
     </row>
     <row r="170" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF170" s="9"/>
-      <c r="AJ170" s="12"/>
+      <c r="AG170" s="9"/>
+      <c r="AH170" s="15"/>
+      <c r="AI170" s="10"/>
     </row>
     <row r="171" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF171" s="9"/>
-      <c r="AJ171" s="12"/>
+      <c r="AG171" s="9"/>
+      <c r="AH171" s="15"/>
+      <c r="AI171" s="10"/>
     </row>
     <row r="172" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF172" s="9"/>
-      <c r="AJ172" s="12"/>
+      <c r="AG172" s="9"/>
+      <c r="AH172" s="15"/>
+      <c r="AI172" s="10"/>
     </row>
     <row r="173" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF173" s="9"/>
       <c r="AG173" s="9"/>
-      <c r="AH173" s="9"/>
+      <c r="AH173" s="15"/>
       <c r="AI173" s="10"/>
     </row>
     <row r="174" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF174" s="9"/>
       <c r="AG174" s="9"/>
-      <c r="AH174" s="9"/>
+      <c r="AH174" s="15"/>
       <c r="AI174" s="10"/>
     </row>
     <row r="175" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF175" s="9"/>
       <c r="AG175" s="9"/>
-      <c r="AH175" s="9"/>
+      <c r="AH175" s="15"/>
       <c r="AI175" s="10"/>
     </row>
     <row r="176" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF176" s="9"/>
-      <c r="AJ176" s="12"/>
-    </row>
-    <row r="177" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG176" s="9"/>
+      <c r="AH176" s="15"/>
+      <c r="AI176" s="10"/>
+    </row>
+    <row r="177" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF177" s="9"/>
-      <c r="AJ177" s="12"/>
-    </row>
-    <row r="178" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG177" s="9"/>
+      <c r="AH177" s="15"/>
+      <c r="AI177" s="10"/>
+    </row>
+    <row r="178" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF178" s="9"/>
-      <c r="AJ178" s="12"/>
-    </row>
-    <row r="179" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG178" s="9"/>
+      <c r="AH178" s="15"/>
+      <c r="AI178" s="10"/>
+    </row>
+    <row r="179" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF179" s="9"/>
-      <c r="AJ179" s="12"/>
-    </row>
-    <row r="180" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG179" s="9"/>
+      <c r="AH179" s="15"/>
+      <c r="AI179" s="10"/>
+    </row>
+    <row r="180" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF180" s="9"/>
-      <c r="AJ180" s="12"/>
-    </row>
-    <row r="181" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG180" s="9"/>
+      <c r="AH180" s="15"/>
+      <c r="AI180" s="10"/>
+    </row>
+    <row r="181" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF181" s="9"/>
-      <c r="AJ181" s="12"/>
-    </row>
-    <row r="182" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG181" s="9"/>
+      <c r="AH181" s="15"/>
+      <c r="AI181" s="10"/>
+    </row>
+    <row r="182" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF182" s="9"/>
-      <c r="AJ182" s="12"/>
-    </row>
-    <row r="183" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG182" s="9"/>
+      <c r="AH182" s="15"/>
+      <c r="AI182" s="10"/>
+    </row>
+    <row r="183" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF183" s="9"/>
-      <c r="AJ183" s="12"/>
-    </row>
-    <row r="184" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG183" s="9"/>
+      <c r="AH183" s="15"/>
+      <c r="AI183" s="10"/>
+    </row>
+    <row r="184" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF184" s="9"/>
-      <c r="AJ184" s="12"/>
-    </row>
-    <row r="185" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AG184" s="9"/>
+      <c r="AH184" s="15"/>
+      <c r="AI184" s="10"/>
+    </row>
+    <row r="185" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF185" s="9"/>
       <c r="AG185" s="9"/>
-      <c r="AH185" s="9"/>
+      <c r="AH185" s="15"/>
       <c r="AI185" s="10"/>
     </row>
-    <row r="186" spans="32:36" x14ac:dyDescent="0.3">
+    <row r="186" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF186" s="9"/>
       <c r="AG186" s="9"/>
-      <c r="AH186" s="9"/>
+      <c r="AH186" s="15"/>
       <c r="AI186" s="10"/>
     </row>
-    <row r="187" spans="32:36" x14ac:dyDescent="0.3">
+    <row r="187" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF187" s="9"/>
       <c r="AG187" s="9"/>
-      <c r="AH187" s="9"/>
+      <c r="AH187" s="15"/>
       <c r="AI187" s="10"/>
     </row>
-    <row r="188" spans="32:36" x14ac:dyDescent="0.3">
+    <row r="188" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF188" s="9"/>
       <c r="AG188" s="9"/>
-      <c r="AH188" s="9"/>
+      <c r="AH188" s="15"/>
       <c r="AI188" s="10"/>
     </row>
-    <row r="189" spans="32:36" x14ac:dyDescent="0.3">
+    <row r="189" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF189" s="9"/>
       <c r="AG189" s="9"/>
-      <c r="AH189" s="9"/>
+      <c r="AH189" s="15"/>
       <c r="AI189" s="10"/>
     </row>
-    <row r="190" spans="32:36" x14ac:dyDescent="0.3">
+    <row r="190" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF190" s="9"/>
       <c r="AG190" s="9"/>
-      <c r="AH190" s="9"/>
+      <c r="AH190" s="15"/>
       <c r="AI190" s="10"/>
     </row>
-    <row r="191" spans="32:36" x14ac:dyDescent="0.3">
+    <row r="191" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF191" s="9"/>
       <c r="AG191" s="9"/>
-      <c r="AH191" s="9"/>
+      <c r="AH191" s="15"/>
       <c r="AI191" s="10"/>
     </row>
-    <row r="192" spans="32:36" x14ac:dyDescent="0.3">
+    <row r="192" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF192" s="9"/>
       <c r="AG192" s="9"/>
-      <c r="AH192" s="9"/>
+      <c r="AH192" s="15"/>
       <c r="AI192" s="10"/>
     </row>
     <row r="193" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF193" s="9"/>
       <c r="AG193" s="9"/>
-      <c r="AH193" s="9"/>
+      <c r="AH193" s="15"/>
       <c r="AI193" s="10"/>
     </row>
     <row r="194" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF194" s="9"/>
       <c r="AG194" s="9"/>
-      <c r="AH194" s="9"/>
+      <c r="AH194" s="15"/>
       <c r="AI194" s="10"/>
     </row>
     <row r="195" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF195" s="9"/>
       <c r="AG195" s="9"/>
-      <c r="AH195" s="9"/>
+      <c r="AH195" s="15"/>
       <c r="AI195" s="10"/>
     </row>
     <row r="196" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF196" s="9"/>
       <c r="AG196" s="9"/>
-      <c r="AH196" s="9"/>
+      <c r="AH196" s="15"/>
       <c r="AI196" s="10"/>
     </row>
     <row r="197" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF197" s="9"/>
       <c r="AG197" s="9"/>
-      <c r="AH197" s="9"/>
+      <c r="AH197" s="15"/>
       <c r="AI197" s="10"/>
     </row>
     <row r="198" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF198" s="9"/>
       <c r="AG198" s="9"/>
-      <c r="AH198" s="9"/>
+      <c r="AH198" s="15"/>
       <c r="AI198" s="10"/>
     </row>
     <row r="199" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF199" s="9"/>
       <c r="AG199" s="9"/>
-      <c r="AH199" s="9"/>
+      <c r="AH199" s="15"/>
       <c r="AI199" s="10"/>
     </row>
     <row r="200" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF200" s="9"/>
       <c r="AG200" s="9"/>
-      <c r="AH200" s="9"/>
+      <c r="AH200" s="15"/>
       <c r="AI200" s="10"/>
     </row>
     <row r="201" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF201" s="9"/>
       <c r="AG201" s="9"/>
-      <c r="AH201" s="9"/>
+      <c r="AH201" s="15"/>
       <c r="AI201" s="10"/>
     </row>
     <row r="202" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF202" s="9"/>
       <c r="AG202" s="9"/>
-      <c r="AH202" s="9"/>
+      <c r="AH202" s="15"/>
       <c r="AI202" s="10"/>
     </row>
     <row r="203" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF203" s="9"/>
       <c r="AG203" s="9"/>
-      <c r="AH203" s="9"/>
+      <c r="AH203" s="15"/>
       <c r="AI203" s="10"/>
     </row>
     <row r="204" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF204" s="9"/>
       <c r="AG204" s="9"/>
-      <c r="AH204" s="9"/>
+      <c r="AH204" s="15"/>
       <c r="AI204" s="10"/>
     </row>
     <row r="205" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF205" s="9"/>
       <c r="AG205" s="9"/>
-      <c r="AH205" s="9"/>
+      <c r="AH205" s="15"/>
       <c r="AI205" s="10"/>
     </row>
     <row r="206" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF206" s="9"/>
       <c r="AG206" s="9"/>
-      <c r="AH206" s="9"/>
+      <c r="AH206" s="15"/>
       <c r="AI206" s="10"/>
     </row>
     <row r="207" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF207" s="9"/>
       <c r="AG207" s="9"/>
-      <c r="AH207" s="9"/>
+      <c r="AH207" s="15"/>
       <c r="AI207" s="10"/>
     </row>
     <row r="208" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF208" s="9"/>
       <c r="AG208" s="9"/>
-      <c r="AH208" s="9"/>
+      <c r="AH208" s="15"/>
       <c r="AI208" s="10"/>
     </row>
     <row r="209" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF209" s="9"/>
       <c r="AG209" s="9"/>
-      <c r="AH209" s="9"/>
+      <c r="AH209" s="15"/>
       <c r="AI209" s="10"/>
     </row>
     <row r="210" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF210" s="9"/>
       <c r="AG210" s="9"/>
-      <c r="AH210" s="9"/>
+      <c r="AH210" s="15"/>
       <c r="AI210" s="10"/>
     </row>
     <row r="211" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF211" s="9"/>
       <c r="AG211" s="9"/>
-      <c r="AH211" s="9"/>
+      <c r="AH211" s="15"/>
       <c r="AI211" s="10"/>
     </row>
     <row r="212" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF212" s="9"/>
       <c r="AG212" s="9"/>
-      <c r="AH212" s="9"/>
+      <c r="AH212" s="15"/>
       <c r="AI212" s="10"/>
     </row>
     <row r="213" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF213" s="9"/>
       <c r="AG213" s="9"/>
-      <c r="AH213" s="9"/>
+      <c r="AH213" s="15"/>
       <c r="AI213" s="10"/>
     </row>
     <row r="214" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF214" s="9"/>
       <c r="AG214" s="9"/>
-      <c r="AH214" s="9"/>
+      <c r="AH214" s="15"/>
       <c r="AI214" s="10"/>
     </row>
     <row r="215" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF215" s="9"/>
       <c r="AG215" s="9"/>
-      <c r="AH215" s="9"/>
+      <c r="AH215" s="15"/>
       <c r="AI215" s="10"/>
     </row>
     <row r="216" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF216" s="9"/>
       <c r="AG216" s="9"/>
-      <c r="AH216" s="9"/>
+      <c r="AH216" s="15"/>
       <c r="AI216" s="10"/>
     </row>
     <row r="217" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF217" s="9"/>
       <c r="AG217" s="9"/>
-      <c r="AH217" s="9"/>
+      <c r="AH217" s="15"/>
       <c r="AI217" s="10"/>
     </row>
     <row r="218" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF218" s="9"/>
       <c r="AG218" s="9"/>
-      <c r="AH218" s="9"/>
+      <c r="AH218" s="15"/>
       <c r="AI218" s="10"/>
     </row>
     <row r="219" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF219" s="9"/>
       <c r="AG219" s="9"/>
-      <c r="AH219" s="9"/>
+      <c r="AH219" s="15"/>
       <c r="AI219" s="10"/>
     </row>
     <row r="220" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF220" s="9"/>
       <c r="AG220" s="9"/>
-      <c r="AH220" s="9"/>
+      <c r="AH220" s="15"/>
       <c r="AI220" s="10"/>
     </row>
     <row r="221" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF221" s="9"/>
       <c r="AG221" s="9"/>
-      <c r="AH221" s="9"/>
+      <c r="AH221" s="15"/>
       <c r="AI221" s="10"/>
     </row>
     <row r="222" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF222" s="9"/>
       <c r="AG222" s="9"/>
-      <c r="AH222" s="9"/>
+      <c r="AH222" s="15"/>
       <c r="AI222" s="10"/>
     </row>
     <row r="223" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF223" s="9"/>
       <c r="AG223" s="9"/>
-      <c r="AH223" s="9"/>
+      <c r="AH223" s="15"/>
       <c r="AI223" s="10"/>
     </row>
     <row r="224" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF224" s="9"/>
       <c r="AG224" s="9"/>
-      <c r="AH224" s="9"/>
+      <c r="AH224" s="15"/>
       <c r="AI224" s="10"/>
     </row>
     <row r="225" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF225" s="9"/>
       <c r="AG225" s="9"/>
-      <c r="AH225" s="9"/>
+      <c r="AH225" s="15"/>
       <c r="AI225" s="10"/>
     </row>
     <row r="226" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF226" s="9"/>
       <c r="AG226" s="9"/>
-      <c r="AH226" s="9"/>
+      <c r="AH226" s="15"/>
       <c r="AI226" s="10"/>
     </row>
     <row r="227" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF227" s="9"/>
       <c r="AG227" s="9"/>
-      <c r="AH227" s="9"/>
+      <c r="AH227" s="15"/>
       <c r="AI227" s="10"/>
     </row>
     <row r="228" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF228" s="9"/>
       <c r="AG228" s="9"/>
-      <c r="AH228" s="9"/>
+      <c r="AH228" s="15"/>
       <c r="AI228" s="10"/>
     </row>
     <row r="229" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF229" s="9"/>
       <c r="AG229" s="9"/>
-      <c r="AH229" s="9"/>
+      <c r="AH229" s="15"/>
       <c r="AI229" s="10"/>
     </row>
     <row r="230" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF230" s="9"/>
       <c r="AG230" s="9"/>
-      <c r="AH230" s="9"/>
+      <c r="AH230" s="15"/>
       <c r="AI230" s="10"/>
     </row>
     <row r="231" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF231" s="9"/>
       <c r="AG231" s="9"/>
-      <c r="AH231" s="9"/>
+      <c r="AH231" s="15"/>
       <c r="AI231" s="10"/>
     </row>
     <row r="232" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF232" s="9"/>
       <c r="AG232" s="9"/>
-      <c r="AH232" s="9"/>
+      <c r="AH232" s="15"/>
       <c r="AI232" s="10"/>
     </row>
     <row r="233" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF233" s="9"/>
       <c r="AG233" s="9"/>
-      <c r="AH233" s="9"/>
+      <c r="AH233" s="15"/>
       <c r="AI233" s="10"/>
     </row>
     <row r="234" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF234" s="9"/>
       <c r="AG234" s="9"/>
-      <c r="AH234" s="9"/>
+      <c r="AH234" s="15"/>
       <c r="AI234" s="10"/>
     </row>
     <row r="235" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF235" s="9"/>
       <c r="AG235" s="9"/>
-      <c r="AH235" s="9"/>
+      <c r="AH235" s="15"/>
       <c r="AI235" s="10"/>
     </row>
     <row r="236" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF236" s="9"/>
       <c r="AG236" s="9"/>
-      <c r="AH236" s="9"/>
+      <c r="AH236" s="15"/>
       <c r="AI236" s="10"/>
     </row>
     <row r="237" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF237" s="9"/>
       <c r="AG237" s="9"/>
-      <c r="AH237" s="9"/>
+      <c r="AH237" s="15"/>
       <c r="AI237" s="10"/>
     </row>
     <row r="238" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF238" s="9"/>
       <c r="AG238" s="9"/>
-      <c r="AH238" s="9"/>
+      <c r="AH238" s="15"/>
       <c r="AI238" s="10"/>
     </row>
     <row r="239" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF239" s="9"/>
       <c r="AG239" s="9"/>
-      <c r="AH239" s="9"/>
+      <c r="AH239" s="15"/>
       <c r="AI239" s="10"/>
     </row>
     <row r="240" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF240" s="9"/>
       <c r="AG240" s="9"/>
-      <c r="AH240" s="9"/>
+      <c r="AH240" s="15"/>
       <c r="AI240" s="10"/>
     </row>
     <row r="241" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF241" s="9"/>
       <c r="AG241" s="9"/>
-      <c r="AH241" s="9"/>
+      <c r="AH241" s="15"/>
       <c r="AI241" s="10"/>
     </row>
     <row r="242" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF242" s="9"/>
       <c r="AG242" s="9"/>
-      <c r="AH242" s="9"/>
+      <c r="AH242" s="15"/>
       <c r="AI242" s="10"/>
     </row>
     <row r="243" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF243" s="9"/>
       <c r="AG243" s="9"/>
-      <c r="AH243" s="9"/>
+      <c r="AH243" s="15"/>
       <c r="AI243" s="10"/>
     </row>
     <row r="244" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF244" s="9"/>
       <c r="AG244" s="9"/>
-      <c r="AH244" s="9"/>
+      <c r="AH244" s="15"/>
       <c r="AI244" s="10"/>
     </row>
     <row r="245" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF245" s="9"/>
       <c r="AG245" s="9"/>
-      <c r="AH245" s="9"/>
+      <c r="AH245" s="15"/>
       <c r="AI245" s="10"/>
     </row>
     <row r="246" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF246" s="9"/>
       <c r="AG246" s="9"/>
-      <c r="AH246" s="9"/>
+      <c r="AH246" s="15"/>
       <c r="AI246" s="10"/>
     </row>
     <row r="247" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF247" s="9"/>
       <c r="AG247" s="9"/>
-      <c r="AH247" s="9"/>
+      <c r="AH247" s="15"/>
       <c r="AI247" s="10"/>
     </row>
     <row r="248" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF248" s="9"/>
       <c r="AG248" s="9"/>
-      <c r="AH248" s="9"/>
+      <c r="AH248" s="15"/>
       <c r="AI248" s="10"/>
     </row>
     <row r="249" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF249" s="9"/>
       <c r="AG249" s="9"/>
-      <c r="AH249" s="9"/>
+      <c r="AH249" s="15"/>
       <c r="AI249" s="10"/>
     </row>
     <row r="250" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF250" s="9"/>
       <c r="AG250" s="9"/>
-      <c r="AH250" s="9"/>
+      <c r="AH250" s="15"/>
       <c r="AI250" s="10"/>
     </row>
     <row r="251" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF251" s="9"/>
       <c r="AG251" s="9"/>
-      <c r="AH251" s="9"/>
+      <c r="AH251" s="15"/>
       <c r="AI251" s="10"/>
     </row>
     <row r="252" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF252" s="9"/>
       <c r="AG252" s="9"/>
-      <c r="AH252" s="9"/>
+      <c r="AH252" s="15"/>
       <c r="AI252" s="10"/>
     </row>
     <row r="253" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF253" s="9"/>
       <c r="AG253" s="9"/>
-      <c r="AH253" s="9"/>
+      <c r="AH253" s="15"/>
       <c r="AI253" s="10"/>
     </row>
     <row r="254" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF254" s="9"/>
       <c r="AG254" s="9"/>
-      <c r="AH254" s="9"/>
+      <c r="AH254" s="15"/>
       <c r="AI254" s="10"/>
     </row>
     <row r="255" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF255" s="9"/>
       <c r="AG255" s="9"/>
-      <c r="AH255" s="9"/>
+      <c r="AH255" s="15"/>
       <c r="AI255" s="10"/>
     </row>
     <row r="256" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF256" s="9"/>
       <c r="AG256" s="9"/>
-      <c r="AH256" s="9"/>
+      <c r="AH256" s="15"/>
       <c r="AI256" s="10"/>
     </row>
-    <row r="257" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="257" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF257" s="9"/>
       <c r="AG257" s="9"/>
-      <c r="AH257" s="9"/>
+      <c r="AH257" s="15"/>
       <c r="AI257" s="10"/>
     </row>
-    <row r="258" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="258" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF258" s="9"/>
       <c r="AG258" s="9"/>
-      <c r="AH258" s="9"/>
+      <c r="AH258" s="15"/>
       <c r="AI258" s="10"/>
     </row>
-    <row r="259" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="259" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF259" s="9"/>
       <c r="AG259" s="9"/>
-      <c r="AH259" s="9"/>
+      <c r="AH259" s="15"/>
       <c r="AI259" s="10"/>
     </row>
-    <row r="260" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="260" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF260" s="9"/>
       <c r="AG260" s="9"/>
-      <c r="AH260" s="9"/>
+      <c r="AH260" s="15"/>
       <c r="AI260" s="10"/>
     </row>
-    <row r="261" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="261" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF261" s="9"/>
       <c r="AG261" s="9"/>
-      <c r="AH261" s="9"/>
+      <c r="AH261" s="15"/>
       <c r="AI261" s="10"/>
     </row>
-    <row r="262" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="262" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF262" s="9"/>
       <c r="AG262" s="9"/>
-      <c r="AH262" s="9"/>
+      <c r="AH262" s="15"/>
       <c r="AI262" s="10"/>
     </row>
-    <row r="263" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="263" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF263" s="9"/>
       <c r="AG263" s="9"/>
-      <c r="AH263" s="9"/>
+      <c r="AH263" s="15"/>
       <c r="AI263" s="10"/>
     </row>
-    <row r="264" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="264" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF264" s="9"/>
       <c r="AG264" s="9"/>
-      <c r="AH264" s="9"/>
+      <c r="AH264" s="15"/>
       <c r="AI264" s="10"/>
     </row>
-    <row r="265" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="265" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF265" s="9"/>
       <c r="AG265" s="9"/>
-      <c r="AH265" s="9"/>
+      <c r="AH265" s="15"/>
       <c r="AI265" s="10"/>
     </row>
-    <row r="266" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="266" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF266" s="9"/>
       <c r="AG266" s="9"/>
-      <c r="AH266" s="9"/>
+      <c r="AH266" s="15"/>
       <c r="AI266" s="10"/>
     </row>
-    <row r="267" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="267" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF267" s="9"/>
       <c r="AG267" s="9"/>
-      <c r="AH267" s="9"/>
+      <c r="AH267" s="15"/>
       <c r="AI267" s="10"/>
     </row>
-    <row r="268" spans="32:35" x14ac:dyDescent="0.3">
+    <row r="268" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF268" s="9"/>
-      <c r="AG268" s="9"/>
-      <c r="AH268" s="9"/>
-      <c r="AI268" s="10"/>
-    </row>
-    <row r="269" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ268" s="12"/>
+    </row>
+    <row r="269" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF269" s="9"/>
-      <c r="AG269" s="9"/>
-      <c r="AH269" s="9"/>
-      <c r="AI269" s="10"/>
-    </row>
-    <row r="270" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ269" s="12"/>
+    </row>
+    <row r="270" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF270" s="9"/>
-      <c r="AG270" s="9"/>
-      <c r="AH270" s="9"/>
-      <c r="AI270" s="10"/>
-    </row>
-    <row r="271" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ270" s="12"/>
+    </row>
+    <row r="271" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF271" s="9"/>
-      <c r="AG271" s="9"/>
-      <c r="AH271" s="9"/>
-      <c r="AI271" s="10"/>
-    </row>
-    <row r="272" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ271" s="12"/>
+    </row>
+    <row r="272" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF272" s="9"/>
-      <c r="AG272" s="9"/>
-      <c r="AH272" s="9"/>
-      <c r="AI272" s="10"/>
-    </row>
-    <row r="273" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ272" s="12"/>
+    </row>
+    <row r="273" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF273" s="9"/>
-      <c r="AG273" s="9"/>
-      <c r="AH273" s="9"/>
-      <c r="AI273" s="10"/>
-    </row>
-    <row r="274" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ273" s="12"/>
+    </row>
+    <row r="274" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF274" s="9"/>
-      <c r="AG274" s="9"/>
-      <c r="AH274" s="9"/>
-      <c r="AI274" s="10"/>
-    </row>
-    <row r="275" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AJ274" s="12"/>
+    </row>
+    <row r="275" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF275" s="9"/>
-      <c r="AG275" s="9"/>
-      <c r="AH275" s="9"/>
-      <c r="AI275" s="10"/>
-    </row>
-    <row r="276" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG275" s="13"/>
+      <c r="AH275" s="26"/>
+      <c r="AI275" s="14"/>
+      <c r="AJ275" s="14"/>
+    </row>
+    <row r="276" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF276" s="9"/>
-      <c r="AG276" s="9"/>
-      <c r="AH276" s="9"/>
-      <c r="AI276" s="10"/>
-    </row>
-    <row r="277" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG276" s="13"/>
+      <c r="AH276" s="26"/>
+      <c r="AI276" s="14"/>
+      <c r="AJ276" s="14"/>
+    </row>
+    <row r="277" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF277" s="9"/>
-      <c r="AG277" s="9"/>
-      <c r="AH277" s="9"/>
-      <c r="AI277" s="10"/>
-    </row>
-    <row r="278" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG277" s="13"/>
+      <c r="AH277" s="26"/>
+      <c r="AI277" s="14"/>
+      <c r="AJ277" s="14"/>
+    </row>
+    <row r="278" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF278" s="9"/>
-      <c r="AG278" s="9"/>
-      <c r="AH278" s="9"/>
-      <c r="AI278" s="10"/>
-    </row>
-    <row r="279" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG278" s="13"/>
+      <c r="AH278" s="26"/>
+      <c r="AI278" s="14"/>
+      <c r="AJ278" s="14"/>
+    </row>
+    <row r="279" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF279" s="9"/>
-      <c r="AG279" s="9"/>
-      <c r="AH279" s="9"/>
-      <c r="AI279" s="10"/>
-    </row>
-    <row r="280" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG279" s="13"/>
+      <c r="AH279" s="26"/>
+      <c r="AI279" s="14"/>
+      <c r="AJ279" s="14"/>
+    </row>
+    <row r="280" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF280" s="9"/>
-      <c r="AG280" s="9"/>
-      <c r="AH280" s="9"/>
-      <c r="AI280" s="10"/>
-    </row>
-    <row r="281" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG280" s="13"/>
+      <c r="AH280" s="26"/>
+      <c r="AI280" s="14"/>
+      <c r="AJ280" s="14"/>
+    </row>
+    <row r="281" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF281" s="9"/>
-      <c r="AG281" s="9"/>
-      <c r="AH281" s="9"/>
-      <c r="AI281" s="10"/>
-    </row>
-    <row r="282" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG281" s="13"/>
+      <c r="AH281" s="26"/>
+      <c r="AI281" s="14"/>
+      <c r="AJ281" s="14"/>
+    </row>
+    <row r="282" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF282" s="9"/>
-      <c r="AG282" s="9"/>
-      <c r="AH282" s="9"/>
-      <c r="AI282" s="10"/>
-    </row>
-    <row r="283" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG282" s="13"/>
+      <c r="AH282" s="26"/>
+      <c r="AI282" s="14"/>
+      <c r="AJ282" s="14"/>
+    </row>
+    <row r="283" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF283" s="9"/>
-      <c r="AG283" s="9"/>
-      <c r="AH283" s="9"/>
-      <c r="AI283" s="10"/>
-    </row>
-    <row r="284" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG283" s="13"/>
+      <c r="AH283" s="26"/>
+      <c r="AI283" s="14"/>
+      <c r="AJ283" s="14"/>
+    </row>
+    <row r="284" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF284" s="9"/>
-      <c r="AG284" s="9"/>
-      <c r="AH284" s="9"/>
-      <c r="AI284" s="10"/>
-    </row>
-    <row r="285" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG284" s="13"/>
+      <c r="AH284" s="26"/>
+      <c r="AI284" s="14"/>
+      <c r="AJ284" s="14"/>
+    </row>
+    <row r="285" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF285" s="9"/>
-      <c r="AG285" s="9"/>
-      <c r="AH285" s="9"/>
-      <c r="AI285" s="10"/>
-    </row>
-    <row r="286" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG285" s="13"/>
+      <c r="AH285" s="26"/>
+      <c r="AI285" s="14"/>
+      <c r="AJ285" s="14"/>
+    </row>
+    <row r="286" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF286" s="9"/>
-      <c r="AG286" s="9"/>
-      <c r="AH286" s="9"/>
-      <c r="AI286" s="10"/>
-    </row>
-    <row r="287" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG286" s="13"/>
+      <c r="AH286" s="26"/>
+      <c r="AI286" s="14"/>
+      <c r="AJ286" s="14"/>
+    </row>
+    <row r="287" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF287" s="9"/>
-      <c r="AG287" s="9"/>
-      <c r="AH287" s="9"/>
-      <c r="AI287" s="10"/>
-    </row>
-    <row r="288" spans="32:35" x14ac:dyDescent="0.3">
+      <c r="AG287" s="13"/>
+      <c r="AH287" s="26"/>
+      <c r="AI287" s="14"/>
+      <c r="AJ287" s="14"/>
+    </row>
+    <row r="288" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF288" s="9"/>
-      <c r="AG288" s="9"/>
-      <c r="AH288" s="9"/>
-      <c r="AI288" s="10"/>
+      <c r="AG288" s="13"/>
+      <c r="AH288" s="26"/>
+      <c r="AI288" s="14"/>
+      <c r="AJ288" s="14"/>
     </row>
     <row r="289" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF289" s="9"/>
-      <c r="AJ289" s="12"/>
+      <c r="AG289" s="13"/>
+      <c r="AH289" s="26"/>
+      <c r="AI289" s="14"/>
+      <c r="AJ289" s="14"/>
     </row>
     <row r="290" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF290" s="9"/>
-      <c r="AJ290" s="12"/>
+      <c r="AG290" s="13"/>
+      <c r="AH290" s="26"/>
+      <c r="AI290" s="14"/>
+      <c r="AJ290" s="14"/>
     </row>
     <row r="291" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF291" s="9"/>
-      <c r="AJ291" s="12"/>
+      <c r="AG291" s="13"/>
+      <c r="AH291" s="26"/>
+      <c r="AI291" s="14"/>
+      <c r="AJ291" s="14"/>
     </row>
     <row r="292" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF292" s="9"/>
-      <c r="AJ292" s="12"/>
+      <c r="AG292" s="13"/>
+      <c r="AH292" s="26"/>
+      <c r="AI292" s="14"/>
+      <c r="AJ292" s="14"/>
     </row>
     <row r="293" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF293" s="9"/>
-      <c r="AJ293" s="12"/>
+      <c r="AG293" s="13"/>
+      <c r="AH293" s="26"/>
+      <c r="AI293" s="14"/>
+      <c r="AJ293" s="14"/>
     </row>
     <row r="294" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF294" s="9"/>
-      <c r="AJ294" s="12"/>
+      <c r="AG294" s="13"/>
+      <c r="AH294" s="26"/>
+      <c r="AI294" s="14"/>
+      <c r="AJ294" s="14"/>
     </row>
     <row r="295" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF295" s="9"/>
-      <c r="AJ295" s="12"/>
+      <c r="AG295" s="13"/>
+      <c r="AH295" s="26"/>
+      <c r="AI295" s="14"/>
+      <c r="AJ295" s="14"/>
     </row>
     <row r="296" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF296" s="9"/>
-      <c r="AG296" s="13"/>
-      <c r="AH296" s="13"/>
-      <c r="AI296" s="14"/>
-      <c r="AJ296" s="14"/>
+      <c r="AG296" s="9"/>
+      <c r="AH296" s="15"/>
+      <c r="AI296" s="10"/>
     </row>
     <row r="297" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF297" s="9"/>
-      <c r="AG297" s="13"/>
-      <c r="AH297" s="13"/>
-      <c r="AI297" s="14"/>
-      <c r="AJ297" s="14"/>
+      <c r="AG297" s="9"/>
+      <c r="AH297" s="15"/>
+      <c r="AI297" s="10"/>
     </row>
     <row r="298" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF298" s="9"/>
-      <c r="AG298" s="13"/>
-      <c r="AH298" s="13"/>
-      <c r="AI298" s="14"/>
-      <c r="AJ298" s="14"/>
+      <c r="AG298" s="9"/>
+      <c r="AH298" s="15"/>
+      <c r="AI298" s="10"/>
     </row>
     <row r="299" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF299" s="9"/>
-      <c r="AG299" s="13"/>
-      <c r="AH299" s="13"/>
-      <c r="AI299" s="14"/>
-      <c r="AJ299" s="14"/>
+      <c r="AG299" s="9"/>
+      <c r="AH299" s="15"/>
+      <c r="AI299" s="10"/>
     </row>
     <row r="300" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF300" s="9"/>
-      <c r="AG300" s="13"/>
-      <c r="AH300" s="13"/>
-      <c r="AI300" s="14"/>
-      <c r="AJ300" s="14"/>
+      <c r="AG300" s="9"/>
+      <c r="AH300" s="15"/>
+      <c r="AI300" s="10"/>
     </row>
     <row r="301" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF301" s="9"/>
-      <c r="AG301" s="13"/>
-      <c r="AH301" s="13"/>
-      <c r="AI301" s="14"/>
-      <c r="AJ301" s="14"/>
+      <c r="AG301" s="9"/>
+      <c r="AH301" s="15"/>
+      <c r="AI301" s="10"/>
     </row>
     <row r="302" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF302" s="9"/>
-      <c r="AG302" s="13"/>
-      <c r="AH302" s="13"/>
-      <c r="AI302" s="14"/>
-      <c r="AJ302" s="14"/>
+      <c r="AG302" s="9"/>
+      <c r="AH302" s="15"/>
+      <c r="AI302" s="10"/>
     </row>
     <row r="303" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF303" s="9"/>
-      <c r="AG303" s="13"/>
-      <c r="AH303" s="13"/>
-      <c r="AI303" s="14"/>
-      <c r="AJ303" s="14"/>
+      <c r="AG303" s="9"/>
+      <c r="AH303" s="15"/>
+      <c r="AI303" s="10"/>
     </row>
     <row r="304" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF304" s="9"/>
-      <c r="AG304" s="13"/>
-      <c r="AH304" s="13"/>
-      <c r="AI304" s="14"/>
-      <c r="AJ304" s="14"/>
+      <c r="AG304" s="9"/>
+      <c r="AH304" s="15"/>
+      <c r="AI304" s="10"/>
     </row>
     <row r="305" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF305" s="9"/>
-      <c r="AG305" s="13"/>
-      <c r="AH305" s="13"/>
-      <c r="AI305" s="14"/>
-      <c r="AJ305" s="14"/>
+      <c r="AG305" s="9"/>
+      <c r="AH305" s="15"/>
+      <c r="AI305" s="10"/>
     </row>
     <row r="306" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF306" s="9"/>
-      <c r="AG306" s="13"/>
-      <c r="AH306" s="13"/>
-      <c r="AI306" s="14"/>
+      <c r="AG306" s="9"/>
+      <c r="AH306" s="15"/>
+      <c r="AI306" s="10"/>
       <c r="AJ306" s="14"/>
     </row>
     <row r="307" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF307" s="9"/>
-      <c r="AG307" s="13"/>
-      <c r="AH307" s="13"/>
-      <c r="AI307" s="14"/>
+      <c r="AG307" s="9"/>
+      <c r="AH307" s="15"/>
+      <c r="AI307" s="10"/>
       <c r="AJ307" s="14"/>
     </row>
     <row r="308" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF308" s="9"/>
-      <c r="AG308" s="13"/>
-      <c r="AH308" s="13"/>
-      <c r="AI308" s="14"/>
+      <c r="AG308" s="9"/>
+      <c r="AH308" s="15"/>
+      <c r="AI308" s="10"/>
       <c r="AJ308" s="14"/>
     </row>
     <row r="309" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF309" s="9"/>
       <c r="AG309" s="13"/>
-      <c r="AH309" s="13"/>
+      <c r="AH309" s="26"/>
       <c r="AI309" s="14"/>
       <c r="AJ309" s="14"/>
     </row>
     <row r="310" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF310" s="9"/>
       <c r="AG310" s="13"/>
-      <c r="AH310" s="13"/>
+      <c r="AH310" s="26"/>
       <c r="AI310" s="14"/>
       <c r="AJ310" s="14"/>
     </row>
     <row r="311" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF311" s="9"/>
       <c r="AG311" s="13"/>
-      <c r="AH311" s="13"/>
+      <c r="AH311" s="26"/>
       <c r="AI311" s="14"/>
       <c r="AJ311" s="14"/>
     </row>
     <row r="312" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF312" s="9"/>
       <c r="AG312" s="13"/>
-      <c r="AH312" s="13"/>
+      <c r="AH312" s="26"/>
       <c r="AI312" s="14"/>
       <c r="AJ312" s="14"/>
     </row>
     <row r="313" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF313" s="9"/>
       <c r="AG313" s="13"/>
-      <c r="AH313" s="13"/>
+      <c r="AH313" s="26"/>
       <c r="AI313" s="14"/>
       <c r="AJ313" s="14"/>
     </row>
     <row r="314" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF314" s="9"/>
       <c r="AG314" s="13"/>
-      <c r="AH314" s="13"/>
+      <c r="AH314" s="26"/>
       <c r="AI314" s="14"/>
       <c r="AJ314" s="14"/>
     </row>
     <row r="315" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF315" s="9"/>
       <c r="AG315" s="13"/>
-      <c r="AH315" s="13"/>
+      <c r="AH315" s="26"/>
       <c r="AI315" s="14"/>
       <c r="AJ315" s="14"/>
     </row>
     <row r="316" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF316" s="9"/>
       <c r="AG316" s="13"/>
-      <c r="AH316" s="13"/>
+      <c r="AH316" s="26"/>
       <c r="AI316" s="14"/>
       <c r="AJ316" s="14"/>
     </row>
     <row r="317" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF317" s="9"/>
-      <c r="AG317" s="9"/>
-      <c r="AH317" s="9"/>
-      <c r="AI317" s="10"/>
+      <c r="AG317" s="13"/>
+      <c r="AH317" s="26"/>
+      <c r="AI317" s="14"/>
+      <c r="AJ317" s="14"/>
     </row>
     <row r="318" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF318" s="9"/>
       <c r="AG318" s="9"/>
-      <c r="AH318" s="9"/>
+      <c r="AH318" s="15"/>
       <c r="AI318" s="10"/>
+      <c r="AJ318" s="14"/>
     </row>
     <row r="319" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF319" s="9"/>
-      <c r="AG319" s="9"/>
-      <c r="AH319" s="9"/>
-      <c r="AI319" s="10"/>
+      <c r="AG319" s="13"/>
+      <c r="AH319" s="26"/>
+      <c r="AI319" s="14"/>
+      <c r="AJ319" s="14"/>
     </row>
     <row r="320" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF320" s="9"/>
-      <c r="AG320" s="9"/>
-      <c r="AH320" s="9"/>
-      <c r="AI320" s="10"/>
+      <c r="AG320" s="13"/>
+      <c r="AH320" s="26"/>
+      <c r="AI320" s="14"/>
+      <c r="AJ320" s="14"/>
     </row>
     <row r="321" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF321" s="9"/>
-      <c r="AG321" s="9"/>
-      <c r="AH321" s="9"/>
-      <c r="AI321" s="10"/>
+      <c r="AG321" s="13"/>
+      <c r="AH321" s="26"/>
+      <c r="AI321" s="14"/>
+      <c r="AJ321" s="14"/>
     </row>
     <row r="322" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF322" s="9"/>
-      <c r="AG322" s="9"/>
-      <c r="AH322" s="9"/>
-      <c r="AI322" s="10"/>
+      <c r="AG322" s="13"/>
+      <c r="AH322" s="26"/>
+      <c r="AI322" s="14"/>
+      <c r="AJ322" s="14"/>
     </row>
     <row r="323" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF323" s="9"/>
-      <c r="AG323" s="9"/>
-      <c r="AH323" s="9"/>
-      <c r="AI323" s="10"/>
+      <c r="AG323" s="13"/>
+      <c r="AH323" s="26"/>
+      <c r="AI323" s="14"/>
+      <c r="AJ323" s="14"/>
     </row>
     <row r="324" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF324" s="9"/>
-      <c r="AG324" s="9"/>
-      <c r="AH324" s="9"/>
-      <c r="AI324" s="10"/>
+      <c r="AG324" s="13"/>
+      <c r="AH324" s="26"/>
+      <c r="AI324" s="14"/>
+      <c r="AJ324" s="14"/>
     </row>
     <row r="325" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF325" s="9"/>
-      <c r="AG325" s="9"/>
-      <c r="AH325" s="9"/>
-      <c r="AI325" s="10"/>
+      <c r="AG325" s="13"/>
+      <c r="AH325" s="26"/>
+      <c r="AI325" s="14"/>
+      <c r="AJ325" s="14"/>
     </row>
     <row r="326" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF326" s="9"/>
-      <c r="AG326" s="9"/>
-      <c r="AH326" s="9"/>
-      <c r="AI326" s="10"/>
+      <c r="AG326" s="13"/>
+      <c r="AH326" s="26"/>
+      <c r="AI326" s="14"/>
+      <c r="AJ326" s="14"/>
     </row>
     <row r="327" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF327" s="9"/>
-      <c r="AG327" s="9"/>
-      <c r="AH327" s="9"/>
-      <c r="AI327" s="10"/>
+      <c r="AG327" s="13"/>
+      <c r="AH327" s="26"/>
+      <c r="AI327" s="14"/>
       <c r="AJ327" s="14"/>
     </row>
     <row r="328" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF328" s="9"/>
       <c r="AG328" s="9"/>
-      <c r="AH328" s="9"/>
+      <c r="AH328" s="15"/>
       <c r="AI328" s="10"/>
       <c r="AJ328" s="14"/>
     </row>
     <row r="329" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF329" s="9"/>
       <c r="AG329" s="9"/>
-      <c r="AH329" s="9"/>
+      <c r="AH329" s="15"/>
       <c r="AI329" s="10"/>
       <c r="AJ329" s="14"/>
     </row>
     <row r="330" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF330" s="9"/>
-      <c r="AG330" s="13"/>
-      <c r="AH330" s="13"/>
-      <c r="AI330" s="14"/>
+      <c r="AG330" s="9"/>
+      <c r="AH330" s="15"/>
+      <c r="AI330" s="10"/>
       <c r="AJ330" s="14"/>
     </row>
     <row r="331" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF331" s="9"/>
-      <c r="AG331" s="13"/>
-      <c r="AH331" s="13"/>
-      <c r="AI331" s="14"/>
-      <c r="AJ331" s="14"/>
+      <c r="AG331" s="15"/>
+      <c r="AH331" s="15"/>
+      <c r="AI331" s="16"/>
+      <c r="AJ331" s="16"/>
     </row>
     <row r="332" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF332" s="9"/>
-      <c r="AG332" s="13"/>
-      <c r="AH332" s="13"/>
-      <c r="AI332" s="14"/>
-      <c r="AJ332" s="14"/>
+      <c r="AG332" s="15"/>
+      <c r="AH332" s="15"/>
+      <c r="AI332" s="16"/>
+      <c r="AJ332" s="16"/>
     </row>
     <row r="333" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF333" s="9"/>
-      <c r="AG333" s="13"/>
-      <c r="AH333" s="13"/>
-      <c r="AI333" s="14"/>
-      <c r="AJ333" s="14"/>
+      <c r="AG333" s="15"/>
+      <c r="AH333" s="15"/>
+      <c r="AI333" s="16"/>
+      <c r="AJ333" s="16"/>
     </row>
     <row r="334" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF334" s="9"/>
-      <c r="AG334" s="13"/>
-      <c r="AH334" s="13"/>
-      <c r="AI334" s="14"/>
-      <c r="AJ334" s="14"/>
+      <c r="AG334" s="15"/>
+      <c r="AH334" s="15"/>
+      <c r="AI334" s="16"/>
+      <c r="AJ334" s="16"/>
     </row>
     <row r="335" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF335" s="9"/>
-      <c r="AG335" s="13"/>
-      <c r="AH335" s="13"/>
-      <c r="AI335" s="14"/>
-      <c r="AJ335" s="14"/>
+      <c r="AG335" s="15"/>
+      <c r="AH335" s="15"/>
+      <c r="AI335" s="16"/>
+      <c r="AJ335" s="16"/>
     </row>
     <row r="336" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF336" s="9"/>
-      <c r="AG336" s="13"/>
-      <c r="AH336" s="13"/>
-      <c r="AI336" s="14"/>
-      <c r="AJ336" s="14"/>
+      <c r="AG336" s="15"/>
+      <c r="AH336" s="15"/>
+      <c r="AI336" s="16"/>
+      <c r="AJ336" s="16"/>
     </row>
     <row r="337" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF337" s="9"/>
-      <c r="AG337" s="13"/>
-      <c r="AH337" s="13"/>
-      <c r="AI337" s="14"/>
-      <c r="AJ337" s="14"/>
+      <c r="AG337" s="15"/>
+      <c r="AH337" s="15"/>
+      <c r="AI337" s="16"/>
+      <c r="AJ337" s="16"/>
     </row>
     <row r="338" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF338" s="9"/>
-      <c r="AG338" s="13"/>
-      <c r="AH338" s="13"/>
-      <c r="AI338" s="14"/>
-      <c r="AJ338" s="14"/>
+      <c r="AG338" s="15"/>
+      <c r="AH338" s="15"/>
+      <c r="AI338" s="16"/>
+      <c r="AJ338" s="16"/>
     </row>
     <row r="339" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF339" s="9"/>
       <c r="AG339" s="9"/>
-      <c r="AH339" s="9"/>
+      <c r="AH339" s="15"/>
       <c r="AI339" s="10"/>
       <c r="AJ339" s="14"/>
     </row>
     <row r="340" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF340" s="9"/>
-      <c r="AG340" s="13"/>
-      <c r="AH340" s="13"/>
-      <c r="AI340" s="14"/>
+      <c r="AG340" s="9"/>
+      <c r="AH340" s="15"/>
+      <c r="AI340" s="10"/>
       <c r="AJ340" s="14"/>
     </row>
     <row r="341" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF341" s="9"/>
-      <c r="AG341" s="13"/>
-      <c r="AH341" s="13"/>
-      <c r="AI341" s="14"/>
+      <c r="AG341" s="9"/>
+      <c r="AH341" s="15"/>
+      <c r="AI341" s="10"/>
       <c r="AJ341" s="14"/>
     </row>
     <row r="342" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF342" s="9"/>
-      <c r="AG342" s="13"/>
-      <c r="AH342" s="13"/>
-      <c r="AI342" s="14"/>
-      <c r="AJ342" s="14"/>
+      <c r="AG342" s="9"/>
+      <c r="AH342" s="15"/>
+      <c r="AI342" s="10"/>
     </row>
     <row r="343" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF343" s="9"/>
-      <c r="AG343" s="13"/>
-      <c r="AH343" s="13"/>
-      <c r="AI343" s="14"/>
-      <c r="AJ343" s="14"/>
+      <c r="AG343" s="9"/>
+      <c r="AH343" s="15"/>
+      <c r="AI343" s="10"/>
     </row>
     <row r="344" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF344" s="9"/>
-      <c r="AG344" s="13"/>
-      <c r="AH344" s="13"/>
-      <c r="AI344" s="14"/>
-      <c r="AJ344" s="14"/>
+      <c r="AG344" s="9"/>
+      <c r="AH344" s="15"/>
+      <c r="AI344" s="10"/>
     </row>
     <row r="345" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF345" s="9"/>
-      <c r="AG345" s="13"/>
-      <c r="AH345" s="13"/>
-      <c r="AI345" s="14"/>
-      <c r="AJ345" s="14"/>
+      <c r="AG345" s="9"/>
+      <c r="AH345" s="15"/>
+      <c r="AI345" s="10"/>
     </row>
     <row r="346" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF346" s="9"/>
-      <c r="AG346" s="13"/>
-      <c r="AH346" s="13"/>
-      <c r="AI346" s="14"/>
-      <c r="AJ346" s="14"/>
+      <c r="AG346" s="9"/>
+      <c r="AH346" s="15"/>
+      <c r="AI346" s="10"/>
     </row>
     <row r="347" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF347" s="9"/>
-      <c r="AG347" s="13"/>
-      <c r="AH347" s="13"/>
-      <c r="AI347" s="14"/>
-      <c r="AJ347" s="14"/>
+      <c r="AG347" s="9"/>
+      <c r="AH347" s="15"/>
+      <c r="AI347" s="10"/>
     </row>
     <row r="348" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF348" s="9"/>
-      <c r="AG348" s="13"/>
-      <c r="AH348" s="13"/>
-      <c r="AI348" s="14"/>
-      <c r="AJ348" s="14"/>
+      <c r="AG348" s="9"/>
+      <c r="AH348" s="15"/>
+      <c r="AI348" s="10"/>
     </row>
     <row r="349" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF349" s="9"/>
       <c r="AG349" s="9"/>
-      <c r="AH349" s="9"/>
+      <c r="AH349" s="15"/>
       <c r="AI349" s="10"/>
-      <c r="AJ349" s="14"/>
     </row>
     <row r="350" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF350" s="9"/>
       <c r="AG350" s="9"/>
-      <c r="AH350" s="9"/>
+      <c r="AH350" s="15"/>
       <c r="AI350" s="10"/>
-      <c r="AJ350" s="14"/>
     </row>
     <row r="351" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF351" s="9"/>
       <c r="AG351" s="9"/>
-      <c r="AH351" s="9"/>
+      <c r="AH351" s="15"/>
       <c r="AI351" s="10"/>
-      <c r="AJ351" s="14"/>
     </row>
     <row r="352" spans="32:36" x14ac:dyDescent="0.3">
       <c r="AF352" s="9"/>
-      <c r="AG352" s="15"/>
+      <c r="AG352" s="9"/>
       <c r="AH352" s="15"/>
-      <c r="AI352" s="16"/>
-      <c r="AJ352" s="16"/>
-    </row>
-    <row r="353" spans="32:36" x14ac:dyDescent="0.3">
+      <c r="AI352" s="10"/>
+    </row>
+    <row r="353" spans="32:35" x14ac:dyDescent="0.3">
       <c r="AF353" s="9"/>
-      <c r="AG353" s="15"/>
+      <c r="AG353" s="9"/>
       <c r="AH353" s="15"/>
-      <c r="AI353" s="16"/>
-      <c r="AJ353" s="16"/>
-    </row>
-    <row r="354" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF354" s="9"/>
-      <c r="AG354" s="15"/>
-      <c r="AH354" s="15"/>
-      <c r="AI354" s="16"/>
-      <c r="AJ354" s="16"/>
-    </row>
-    <row r="355" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF355" s="9"/>
-      <c r="AG355" s="15"/>
-      <c r="AH355" s="15"/>
-      <c r="AI355" s="16"/>
-      <c r="AJ355" s="16"/>
-    </row>
-    <row r="356" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF356" s="9"/>
-      <c r="AG356" s="15"/>
-      <c r="AH356" s="15"/>
-      <c r="AI356" s="16"/>
-      <c r="AJ356" s="16"/>
-    </row>
-    <row r="357" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF357" s="9"/>
-      <c r="AG357" s="15"/>
-      <c r="AH357" s="15"/>
-      <c r="AI357" s="16"/>
-      <c r="AJ357" s="16"/>
-    </row>
-    <row r="358" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF358" s="9"/>
-      <c r="AG358" s="15"/>
-      <c r="AH358" s="15"/>
-      <c r="AI358" s="16"/>
-      <c r="AJ358" s="16"/>
-    </row>
-    <row r="359" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF359" s="9"/>
-      <c r="AG359" s="15"/>
-      <c r="AH359" s="15"/>
-      <c r="AI359" s="16"/>
-      <c r="AJ359" s="16"/>
-    </row>
-    <row r="360" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF360" s="9"/>
-      <c r="AG360" s="9"/>
-      <c r="AH360" s="9"/>
-      <c r="AI360" s="10"/>
-      <c r="AJ360" s="14"/>
-    </row>
-    <row r="361" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF361" s="9"/>
-      <c r="AG361" s="9"/>
-      <c r="AH361" s="9"/>
-      <c r="AI361" s="10"/>
-      <c r="AJ361" s="14"/>
-    </row>
-    <row r="362" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF362" s="9"/>
-      <c r="AG362" s="9"/>
-      <c r="AH362" s="9"/>
-      <c r="AI362" s="10"/>
-      <c r="AJ362" s="14"/>
-    </row>
-    <row r="363" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF363" s="9"/>
-      <c r="AG363" s="9"/>
-      <c r="AH363" s="9"/>
-      <c r="AI363" s="10"/>
-    </row>
-    <row r="364" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF364" s="9"/>
-      <c r="AG364" s="9"/>
-      <c r="AH364" s="9"/>
-      <c r="AI364" s="10"/>
-    </row>
-    <row r="365" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF365" s="9"/>
-      <c r="AG365" s="9"/>
-      <c r="AH365" s="9"/>
-      <c r="AI365" s="10"/>
-    </row>
-    <row r="366" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF366" s="9"/>
-      <c r="AG366" s="9"/>
-      <c r="AH366" s="9"/>
-      <c r="AI366" s="10"/>
-    </row>
-    <row r="367" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF367" s="9"/>
-      <c r="AG367" s="9"/>
-      <c r="AH367" s="9"/>
-      <c r="AI367" s="10"/>
-    </row>
-    <row r="368" spans="32:36" x14ac:dyDescent="0.3">
-      <c r="AF368" s="9"/>
-      <c r="AG368" s="9"/>
-      <c r="AH368" s="9"/>
-      <c r="AI368" s="10"/>
-    </row>
-    <row r="369" spans="32:35" x14ac:dyDescent="0.3">
-      <c r="AF369" s="9"/>
-      <c r="AG369" s="9"/>
-      <c r="AH369" s="9"/>
-      <c r="AI369" s="10"/>
-    </row>
-    <row r="370" spans="32:35" x14ac:dyDescent="0.3">
-      <c r="AF370" s="9"/>
-      <c r="AG370" s="9"/>
-      <c r="AH370" s="9"/>
-      <c r="AI370" s="10"/>
-    </row>
-    <row r="371" spans="32:35" x14ac:dyDescent="0.3">
-      <c r="AF371" s="9"/>
-      <c r="AG371" s="9"/>
-      <c r="AH371" s="9"/>
-      <c r="AI371" s="10"/>
-    </row>
-    <row r="372" spans="32:35" x14ac:dyDescent="0.3">
-      <c r="AF372" s="9"/>
-      <c r="AG372" s="9"/>
-      <c r="AH372" s="9"/>
-      <c r="AI372" s="10"/>
-    </row>
-    <row r="373" spans="32:35" x14ac:dyDescent="0.3">
-      <c r="AF373" s="9"/>
-      <c r="AG373" s="9"/>
-      <c r="AH373" s="9"/>
-      <c r="AI373" s="10"/>
-    </row>
-    <row r="374" spans="32:35" x14ac:dyDescent="0.3">
-      <c r="AF374" s="9"/>
-      <c r="AG374" s="9"/>
-      <c r="AH374" s="9"/>
-      <c r="AI374" s="10"/>
+      <c r="AI353" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="AK1:AK2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="AF1:AJ1"/>
@@ -3323,28 +3130,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1ff8efb9-d2f6-48ad-b8a4-78b5e43e4e7a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="26d94f7c-9516-497f-8877-d2bab8403892" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="文档" ma:contentTypeID="0x010100EA249B9729C14C4DACCEF63B96392FF1" ma:contentTypeVersion="20" ma:contentTypeDescription="新建文档。" ma:contentTypeScope="" ma:versionID="7802887b034bb0488cc56512c688a915">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="1ff8efb9-d2f6-48ad-b8a4-78b5e43e4e7a" xmlns:ns3="26d94f7c-9516-497f-8877-d2bab8403892" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f399310843be2bcf5906b5e60b5dcd9e" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3610,29 +3395,29 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C627E8D3-C2E1-47CF-BF02-023F8788D528}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6483D7D9-B9B0-433D-8A2A-BDB69F0E89F4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4f748bf7-a05c-48de-a060-89a2e7e8d9a6"/>
-    <ds:schemaRef ds:uri="de63cf20-70c1-4029-9219-e0d227e15929"/>
-    <ds:schemaRef ds:uri="1ff8efb9-d2f6-48ad-b8a4-78b5e43e4e7a"/>
-    <ds:schemaRef ds:uri="26d94f7c-9516-497f-8877-d2bab8403892"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1ff8efb9-d2f6-48ad-b8a4-78b5e43e4e7a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="26d94f7c-9516-497f-8877-d2bab8403892" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69B9EA-3123-4A3D-8A25-E3F3D95C556B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3650,4 +3435,26 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C627E8D3-C2E1-47CF-BF02-023F8788D528}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6483D7D9-B9B0-433D-8A2A-BDB69F0E89F4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4f748bf7-a05c-48de-a060-89a2e7e8d9a6"/>
+    <ds:schemaRef ds:uri="de63cf20-70c1-4029-9219-e0d227e15929"/>
+    <ds:schemaRef ds:uri="1ff8efb9-d2f6-48ad-b8a4-78b5e43e4e7a"/>
+    <ds:schemaRef ds:uri="26d94f7c-9516-497f-8877-d2bab8403892"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>